<commit_message>
feat: added User.key property as the actual key for the user, instead of email that is not always available. Email and name still exist as optional properties feat: IDP configuration now has a claim_map property that can map existing claims to a new name, e.g. email to __key__ in the example, so that across IDPs the same claim (after mapping) can be used as the key test: launch configs and corresponding test paths/names updated for consistency; test.end_to_end configs added fix: seqdb/omopdb.domain.service.abac class variables fixed test: end_to_end casedb_seqdb_connection fixed to be platform-independent test: casedb.unit.seqdb_remote_app test fixed
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5171D89E-DF80-437B-94F2-667AC7209E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3015D13F-CAF7-4AE5-96AB-84C4E7B328CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="11" activeTab="24" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2409" uniqueCount="874">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="875">
   <si>
     <t>id</t>
   </si>
@@ -2744,6 +2744,9 @@
   </si>
   <si>
     <t>019542cc-8225-8f5d-fa30-d9c3f2629703</t>
+  </si>
+  <si>
+    <t>key</t>
   </si>
 </sst>
 </file>
@@ -3527,1001 +3530,1086 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1200-000000000000}">
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="27" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>874</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>281</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>217</v>
       </c>
       <c r="B2" t="s">
         <v>758</v>
       </c>
-      <c r="C2" s="6" t="str">
-        <f>LEFT($B2,LEN($B2)-9)</f>
+      <c r="C2" t="s">
+        <v>758</v>
+      </c>
+      <c r="D2" s="6" t="str">
+        <f>LEFT($C2,LEN($C2)-9)</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>218</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
         <v>45743.390918726589</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>275</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>873</v>
       </c>
-      <c r="H2" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G2,User!$A:$A,0))</f>
+      <c r="I2" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H2,User!$A:$A,0))</f>
         <v>root1_1</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I2,Organization!$A:$A,0))</f>
+      <c r="K2" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J2,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>219</v>
       </c>
       <c r="B3" s="20" t="s">
         <v>759</v>
       </c>
-      <c r="C3" s="6" t="str">
-        <f t="shared" ref="C3:C28" si="0">LEFT($B3,LEN($B3)-9)</f>
+      <c r="C3" s="20" t="s">
+        <v>759</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <f t="shared" ref="D3:D28" si="0">LEFT($C3,LEN($C3)-9)</f>
         <v>refdata_admin1_1</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>220</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3" s="2">
         <v>45743.390918741461</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>304</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>192</v>
       </c>
-      <c r="H3" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G3,User!$A:$A,0))</f>
+      <c r="I3" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H3,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>43</v>
       </c>
-      <c r="J3" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I3,Organization!$A:$A,0))</f>
+      <c r="K3" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J3,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>221</v>
       </c>
       <c r="B4" t="s">
         <v>760</v>
       </c>
-      <c r="C4" s="6" t="str">
+      <c r="C4" t="s">
+        <v>760</v>
+      </c>
+      <c r="D4" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin1_1</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>222</v>
       </c>
-      <c r="E4" s="2">
+      <c r="F4" s="2">
         <v>45743.390918746562</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>276</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>192</v>
       </c>
-      <c r="H4" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G4,User!$A:$A,0))</f>
+      <c r="I4" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H4,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>43</v>
       </c>
-      <c r="J4" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I4,Organization!$A:$A,0))</f>
+      <c r="K4" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J4,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>223</v>
       </c>
       <c r="B5" t="s">
         <v>761</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" t="s">
+        <v>761</v>
+      </c>
+      <c r="D5" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin2_1</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>224</v>
       </c>
-      <c r="E5" s="2">
+      <c r="F5" s="2">
         <v>45743.390918763551</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>276</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>192</v>
       </c>
-      <c r="H5" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G5,User!$A:$A,0))</f>
+      <c r="I5" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H5,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>46</v>
       </c>
-      <c r="J5" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I5,Organization!$A:$A,0))</f>
+      <c r="K5" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J5,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>225</v>
       </c>
       <c r="B6" t="s">
         <v>762</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" t="s">
+        <v>762</v>
+      </c>
+      <c r="D6" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin3_1</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>226</v>
       </c>
-      <c r="E6" s="2">
+      <c r="F6" s="2">
         <v>45743.390918772537</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>276</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>192</v>
       </c>
-      <c r="H6" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G6,User!$A:$A,0))</f>
+      <c r="I6" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H6,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>49</v>
       </c>
-      <c r="J6" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I6,Organization!$A:$A,0))</f>
+      <c r="K6" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J6,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>227</v>
       </c>
       <c r="B7" t="s">
         <v>763</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" t="s">
+        <v>763</v>
+      </c>
+      <c r="D7" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin4_1</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>228</v>
       </c>
-      <c r="E7" s="2">
+      <c r="F7" s="2">
         <v>45743.390918781181</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>276</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>192</v>
       </c>
-      <c r="H7" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G7,User!$A:$A,0))</f>
+      <c r="I7" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H7,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>52</v>
       </c>
-      <c r="J7" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I7,Organization!$A:$A,0))</f>
+      <c r="K7" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J7,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>229</v>
       </c>
       <c r="B8" t="s">
         <v>764</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" t="s">
+        <v>764</v>
+      </c>
+      <c r="D8" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin5_1</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>230</v>
       </c>
-      <c r="E8" s="2">
+      <c r="F8" s="2">
         <v>45743.3909187889</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>276</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>192</v>
       </c>
-      <c r="H8" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G8,User!$A:$A,0))</f>
+      <c r="I8" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H8,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>55</v>
       </c>
-      <c r="J8" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I8,Organization!$A:$A,0))</f>
+      <c r="K8" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J8,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>231</v>
       </c>
       <c r="B9" t="s">
         <v>765</v>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" t="s">
+        <v>765</v>
+      </c>
+      <c r="D9" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_1</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>232</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F9" s="2">
         <v>45743.390918796598</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>277</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>192</v>
       </c>
-      <c r="H9" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G9,User!$A:$A,0))</f>
+      <c r="I9" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H9,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>43</v>
       </c>
-      <c r="J9" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I9,Organization!$A:$A,0))</f>
+      <c r="K9" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J9,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>233</v>
       </c>
       <c r="B10" t="s">
         <v>766</v>
       </c>
-      <c r="C10" s="6" t="str">
+      <c r="C10" t="s">
+        <v>766</v>
+      </c>
+      <c r="D10" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_2</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>234</v>
       </c>
-      <c r="E10" s="2">
+      <c r="F10" s="2">
         <v>45743.390918801953</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>277</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>192</v>
       </c>
-      <c r="H10" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G10,User!$A:$A,0))</f>
+      <c r="I10" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H10,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>43</v>
       </c>
-      <c r="J10" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I10,Organization!$A:$A,0))</f>
+      <c r="K10" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J10,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>235</v>
       </c>
       <c r="B11" t="s">
         <v>767</v>
       </c>
-      <c r="C11" s="6" t="str">
+      <c r="C11" t="s">
+        <v>767</v>
+      </c>
+      <c r="D11" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_3</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>236</v>
       </c>
-      <c r="E11" s="2">
+      <c r="F11" s="2">
         <v>45743.390918807163</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>277</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>192</v>
       </c>
-      <c r="H11" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G11,User!$A:$A,0))</f>
+      <c r="I11" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H11,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>43</v>
       </c>
-      <c r="J11" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I11,Organization!$A:$A,0))</f>
+      <c r="K11" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J11,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>237</v>
       </c>
       <c r="B12" t="s">
         <v>768</v>
       </c>
-      <c r="C12" s="6" t="str">
+      <c r="C12" t="s">
+        <v>768</v>
+      </c>
+      <c r="D12" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_4</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>238</v>
       </c>
-      <c r="E12" s="2">
+      <c r="F12" s="2">
         <v>45743.3909188123</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>277</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>192</v>
       </c>
-      <c r="H12" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G12,User!$A:$A,0))</f>
+      <c r="I12" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H12,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>43</v>
       </c>
-      <c r="J12" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I12,Organization!$A:$A,0))</f>
+      <c r="K12" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J12,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>239</v>
       </c>
       <c r="B13" t="s">
         <v>769</v>
       </c>
-      <c r="C13" s="6" t="str">
+      <c r="C13" t="s">
+        <v>769</v>
+      </c>
+      <c r="D13" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_1</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>240</v>
       </c>
-      <c r="E13" s="2">
+      <c r="F13" s="2">
         <v>45743.390918817633</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>277</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>192</v>
       </c>
-      <c r="H13" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G13,User!$A:$A,0))</f>
+      <c r="I13" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H13,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>46</v>
       </c>
-      <c r="J13" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I13,Organization!$A:$A,0))</f>
+      <c r="K13" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J13,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>241</v>
       </c>
       <c r="B14" t="s">
         <v>770</v>
       </c>
-      <c r="C14" s="6" t="str">
+      <c r="C14" t="s">
+        <v>770</v>
+      </c>
+      <c r="D14" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_2</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>242</v>
       </c>
-      <c r="E14" s="2">
+      <c r="F14" s="2">
         <v>45743.390918822908</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>277</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>192</v>
       </c>
-      <c r="H14" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G14,User!$A:$A,0))</f>
+      <c r="I14" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H14,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>46</v>
       </c>
-      <c r="J14" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I14,Organization!$A:$A,0))</f>
+      <c r="K14" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J14,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>243</v>
       </c>
       <c r="B15" t="s">
         <v>771</v>
       </c>
-      <c r="C15" s="6" t="str">
+      <c r="C15" t="s">
+        <v>771</v>
+      </c>
+      <c r="D15" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_3</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E15" t="s">
         <v>244</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F15" s="2">
         <v>45743.390918828743</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>277</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>192</v>
       </c>
-      <c r="H15" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G15,User!$A:$A,0))</f>
+      <c r="I15" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H15,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>46</v>
       </c>
-      <c r="J15" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I15,Organization!$A:$A,0))</f>
+      <c r="K15" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J15,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>245</v>
       </c>
       <c r="B16" t="s">
         <v>772</v>
       </c>
-      <c r="C16" s="6" t="str">
+      <c r="C16" t="s">
+        <v>772</v>
+      </c>
+      <c r="D16" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_4</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>246</v>
       </c>
-      <c r="E16" s="2">
+      <c r="F16" s="2">
         <v>45743.390918834302</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>277</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>192</v>
       </c>
-      <c r="H16" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G16,User!$A:$A,0))</f>
+      <c r="I16" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H16,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>46</v>
       </c>
-      <c r="J16" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I16,Organization!$A:$A,0))</f>
+      <c r="K16" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J16,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>247</v>
       </c>
       <c r="B17" t="s">
         <v>773</v>
       </c>
-      <c r="C17" s="6" t="str">
+      <c r="C17" t="s">
+        <v>773</v>
+      </c>
+      <c r="D17" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_1</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>248</v>
       </c>
-      <c r="E17" s="2">
+      <c r="F17" s="2">
         <v>45743.390918839839</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>277</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>192</v>
       </c>
-      <c r="H17" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G17,User!$A:$A,0))</f>
+      <c r="I17" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H17,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>49</v>
       </c>
-      <c r="J17" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I17,Organization!$A:$A,0))</f>
+      <c r="K17" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J17,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>249</v>
       </c>
       <c r="B18" t="s">
         <v>774</v>
       </c>
-      <c r="C18" s="6" t="str">
+      <c r="C18" t="s">
+        <v>774</v>
+      </c>
+      <c r="D18" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_2</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>250</v>
       </c>
-      <c r="E18" s="2">
+      <c r="F18" s="2">
         <v>45743.390918845187</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>277</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>192</v>
       </c>
-      <c r="H18" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G18,User!$A:$A,0))</f>
+      <c r="I18" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H18,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>49</v>
       </c>
-      <c r="J18" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I18,Organization!$A:$A,0))</f>
+      <c r="K18" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J18,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>251</v>
       </c>
       <c r="B19" t="s">
         <v>775</v>
       </c>
-      <c r="C19" s="6" t="str">
+      <c r="C19" t="s">
+        <v>775</v>
+      </c>
+      <c r="D19" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_3</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>252</v>
       </c>
-      <c r="E19" s="2">
+      <c r="F19" s="2">
         <v>45743.390918851088</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>277</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>192</v>
       </c>
-      <c r="H19" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G19,User!$A:$A,0))</f>
+      <c r="I19" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H19,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>49</v>
       </c>
-      <c r="J19" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I19,Organization!$A:$A,0))</f>
+      <c r="K19" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J19,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>253</v>
       </c>
       <c r="B20" t="s">
         <v>776</v>
       </c>
-      <c r="C20" s="6" t="str">
+      <c r="C20" t="s">
+        <v>776</v>
+      </c>
+      <c r="D20" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_4</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>254</v>
       </c>
-      <c r="E20" s="2">
+      <c r="F20" s="2">
         <v>45743.39091885696</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>277</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>192</v>
       </c>
-      <c r="H20" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G20,User!$A:$A,0))</f>
+      <c r="I20" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H20,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>49</v>
       </c>
-      <c r="J20" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I20,Organization!$A:$A,0))</f>
+      <c r="K20" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J20,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>255</v>
       </c>
       <c r="B21" t="s">
         <v>777</v>
       </c>
-      <c r="C21" s="6" t="str">
+      <c r="C21" t="s">
+        <v>777</v>
+      </c>
+      <c r="D21" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_1</v>
       </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>256</v>
       </c>
-      <c r="E21" s="2">
+      <c r="F21" s="2">
         <v>45743.390918862962</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>277</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>192</v>
       </c>
-      <c r="H21" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G21,User!$A:$A,0))</f>
+      <c r="I21" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H21,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>52</v>
       </c>
-      <c r="J21" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I21,Organization!$A:$A,0))</f>
+      <c r="K21" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J21,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>257</v>
       </c>
       <c r="B22" t="s">
         <v>778</v>
       </c>
-      <c r="C22" s="6" t="str">
+      <c r="C22" t="s">
+        <v>778</v>
+      </c>
+      <c r="D22" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_2</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>258</v>
       </c>
-      <c r="E22" s="2">
+      <c r="F22" s="2">
         <v>45743.390918868739</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>277</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>192</v>
       </c>
-      <c r="H22" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G22,User!$A:$A,0))</f>
+      <c r="I22" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H22,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>52</v>
       </c>
-      <c r="J22" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I22,Organization!$A:$A,0))</f>
+      <c r="K22" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J22,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>259</v>
       </c>
       <c r="B23" t="s">
         <v>779</v>
       </c>
-      <c r="C23" s="6" t="str">
+      <c r="C23" t="s">
+        <v>779</v>
+      </c>
+      <c r="D23" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_3</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>260</v>
       </c>
-      <c r="E23" s="2">
+      <c r="F23" s="2">
         <v>45743.390918874728</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>277</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>192</v>
       </c>
-      <c r="H23" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G23,User!$A:$A,0))</f>
+      <c r="I23" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H23,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>52</v>
       </c>
-      <c r="J23" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I23,Organization!$A:$A,0))</f>
+      <c r="K23" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J23,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>261</v>
       </c>
       <c r="B24" t="s">
         <v>780</v>
       </c>
-      <c r="C24" s="6" t="str">
+      <c r="C24" t="s">
+        <v>780</v>
+      </c>
+      <c r="D24" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_4</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>262</v>
       </c>
-      <c r="E24" s="2">
+      <c r="F24" s="2">
         <v>45743.390918881109</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>277</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>192</v>
       </c>
-      <c r="H24" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G24,User!$A:$A,0))</f>
+      <c r="I24" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H24,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>52</v>
       </c>
-      <c r="J24" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I24,Organization!$A:$A,0))</f>
+      <c r="K24" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J24,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>263</v>
       </c>
       <c r="B25" t="s">
         <v>781</v>
       </c>
-      <c r="C25" s="6" t="str">
+      <c r="C25" t="s">
+        <v>781</v>
+      </c>
+      <c r="D25" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_1</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>264</v>
       </c>
-      <c r="E25" s="2">
+      <c r="F25" s="2">
         <v>45743.390918887373</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>277</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>192</v>
       </c>
-      <c r="H25" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G25,User!$A:$A,0))</f>
+      <c r="I25" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H25,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>55</v>
       </c>
-      <c r="J25" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I25,Organization!$A:$A,0))</f>
+      <c r="K25" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J25,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>265</v>
       </c>
       <c r="B26" t="s">
         <v>782</v>
       </c>
-      <c r="C26" s="6" t="str">
+      <c r="C26" t="s">
+        <v>782</v>
+      </c>
+      <c r="D26" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_2</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>266</v>
       </c>
-      <c r="E26" s="2">
+      <c r="F26" s="2">
         <v>45743.39091889358</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>277</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>192</v>
       </c>
-      <c r="H26" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G26,User!$A:$A,0))</f>
+      <c r="I26" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H26,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" t="s">
         <v>55</v>
       </c>
-      <c r="J26" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I26,Organization!$A:$A,0))</f>
+      <c r="K26" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J26,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>267</v>
       </c>
       <c r="B27" t="s">
         <v>783</v>
       </c>
-      <c r="C27" s="6" t="str">
+      <c r="C27" t="s">
+        <v>783</v>
+      </c>
+      <c r="D27" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_3</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>268</v>
       </c>
-      <c r="E27" s="2">
+      <c r="F27" s="2">
         <v>45743.390918900091</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>277</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>192</v>
       </c>
-      <c r="H27" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G27,User!$A:$A,0))</f>
+      <c r="I27" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H27,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>55</v>
       </c>
-      <c r="J27" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I27,Organization!$A:$A,0))</f>
+      <c r="K27" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J27,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>269</v>
       </c>
       <c r="B28" t="s">
         <v>784</v>
       </c>
-      <c r="C28" s="6" t="str">
+      <c r="C28" t="s">
+        <v>784</v>
+      </c>
+      <c r="D28" s="6" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_4</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>270</v>
       </c>
-      <c r="E28" s="2">
+      <c r="F28" s="2">
         <v>45743.390918906553</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>277</v>
       </c>
-      <c r="G28" t="s">
+      <c r="H28" t="s">
         <v>192</v>
       </c>
-      <c r="H28" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($G28,User!$A:$A,0))</f>
+      <c r="I28" s="6" t="str">
+        <f>INDEX(User!$D:$D,MATCH($H28,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>55</v>
       </c>
-      <c r="J28" s="6" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($I28,Organization!$A:$A,0))</f>
+      <c r="K28" s="6" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($J28,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" display="refdata_admin1_1@org1.org" xr:uid="{C6CE08DD-189A-544E-9566-622F7BE1E7EA}"/>
+    <hyperlink ref="C3" r:id="rId1" display="refdata_admin1_1@org1.org" xr:uid="{C6CE08DD-189A-544E-9566-622F7BE1E7EA}"/>
+    <hyperlink ref="B3" r:id="rId2" display="refdata_admin1_1@org1.org" xr:uid="{8DE1F2C7-69F9-4371-8548-F3E32F7DB47B}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11248,7 +11336,7 @@
         <v>873</v>
       </c>
       <c r="D2" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C2,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C2,User!$A:$A,0))</f>
         <v>root1_1</v>
       </c>
       <c r="E2" s="19" t="b">
@@ -11256,11 +11344,11 @@
         <v>1</v>
       </c>
       <c r="F2" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C2,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C2,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G2" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C2,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C2,User!$A:$A,0))</f>
         <v>1</v>
       </c>
       <c r="H2" s="6">
@@ -11342,7 +11430,7 @@
         <v>192</v>
       </c>
       <c r="D3" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C3,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C3,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
       <c r="E3" s="19" t="b">
@@ -11350,11 +11438,11 @@
         <v>1</v>
       </c>
       <c r="F3" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C3,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C3,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G3" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C3,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C3,User!$A:$A,0))</f>
         <v>1</v>
       </c>
       <c r="H3" s="6">
@@ -11436,7 +11524,7 @@
         <v>193</v>
       </c>
       <c r="D4" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C4,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C4,User!$A:$A,0))</f>
         <v>refdata_admin1_1</v>
       </c>
       <c r="E4" s="19" t="b">
@@ -11444,11 +11532,11 @@
         <v>0</v>
       </c>
       <c r="F4" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C4,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C4,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G4" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C4,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C4,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H4" s="6">
@@ -11530,7 +11618,7 @@
         <v>44</v>
       </c>
       <c r="D5" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C5,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C5,User!$A:$A,0))</f>
         <v>org_admin1_1</v>
       </c>
       <c r="E5" s="19" t="b">
@@ -11538,11 +11626,11 @@
         <v>0</v>
       </c>
       <c r="F5" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C5,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C5,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G5" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C5,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C5,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H5" s="6">
@@ -11624,7 +11712,7 @@
         <v>10</v>
       </c>
       <c r="D6" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C6,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C6,User!$A:$A,0))</f>
         <v>org_user1_1</v>
       </c>
       <c r="E6" s="19" t="b">
@@ -11632,11 +11720,11 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C6,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C6,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G6" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C6,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C6,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H6" s="6">
@@ -11718,7 +11806,7 @@
         <v>873</v>
       </c>
       <c r="D7" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C7,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C7,User!$A:$A,0))</f>
         <v>root1_1</v>
       </c>
       <c r="E7" s="19" t="b">
@@ -11726,11 +11814,11 @@
         <v>1</v>
       </c>
       <c r="F7" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C7,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C7,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G7" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C7,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C7,User!$A:$A,0))</f>
         <v>1</v>
       </c>
       <c r="H7" s="6">
@@ -11812,7 +11900,7 @@
         <v>192</v>
       </c>
       <c r="D8" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C8,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C8,User!$A:$A,0))</f>
         <v>app_admin1_1</v>
       </c>
       <c r="E8" s="19" t="b">
@@ -11820,11 +11908,11 @@
         <v>1</v>
       </c>
       <c r="F8" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C8,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C8,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G8" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C8,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C8,User!$A:$A,0))</f>
         <v>1</v>
       </c>
       <c r="H8" s="6">
@@ -11906,7 +11994,7 @@
         <v>44</v>
       </c>
       <c r="D9" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C9,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C9,User!$A:$A,0))</f>
         <v>org_admin1_1</v>
       </c>
       <c r="E9" s="19" t="b">
@@ -11914,11 +12002,11 @@
         <v>0</v>
       </c>
       <c r="F9" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C9,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C9,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G9" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C9,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C9,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H9" s="6">
@@ -12000,7 +12088,7 @@
         <v>47</v>
       </c>
       <c r="D10" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C10,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C10,User!$A:$A,0))</f>
         <v>org_admin2_1</v>
       </c>
       <c r="E10" s="19" t="b">
@@ -12008,11 +12096,11 @@
         <v>0</v>
       </c>
       <c r="F10" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C10,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C10,User!$A:$A,0))</f>
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3</v>
       </c>
       <c r="G10" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C10,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C10,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H10" s="6" t="str">
@@ -12094,7 +12182,7 @@
         <v>50</v>
       </c>
       <c r="D11" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C11,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C11,User!$A:$A,0))</f>
         <v>org_admin3_1</v>
       </c>
       <c r="E11" s="19" t="b">
@@ -12102,11 +12190,11 @@
         <v>0</v>
       </c>
       <c r="F11" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C11,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C11,User!$A:$A,0))</f>
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037</v>
       </c>
       <c r="G11" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C11,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C11,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H11" s="6" t="str">
@@ -12188,7 +12276,7 @@
         <v>53</v>
       </c>
       <c r="D12" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C12,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C12,User!$A:$A,0))</f>
         <v>org_admin4_1</v>
       </c>
       <c r="E12" s="19" t="b">
@@ -12196,11 +12284,11 @@
         <v>0</v>
       </c>
       <c r="F12" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C12,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C12,User!$A:$A,0))</f>
         <v>0195d18c-1c92-d419-4c71-a570f428499b</v>
       </c>
       <c r="G12" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C12,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C12,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H12" s="6" t="str">
@@ -12282,7 +12370,7 @@
         <v>56</v>
       </c>
       <c r="D13" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C13,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C13,User!$A:$A,0))</f>
         <v>org_admin5_1</v>
       </c>
       <c r="E13" s="19" t="b">
@@ -12290,11 +12378,11 @@
         <v>0</v>
       </c>
       <c r="F13" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C13,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C13,User!$A:$A,0))</f>
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0</v>
       </c>
       <c r="G13" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C13,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C13,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H13" s="6" t="str">
@@ -12376,7 +12464,7 @@
         <v>10</v>
       </c>
       <c r="D14" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C14,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C14,User!$A:$A,0))</f>
         <v>org_user1_1</v>
       </c>
       <c r="E14" s="19" t="b">
@@ -12384,11 +12472,11 @@
         <v>1</v>
       </c>
       <c r="F14" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C14,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C14,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G14" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C14,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C14,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H14" s="6">
@@ -12470,7 +12558,7 @@
         <v>12</v>
       </c>
       <c r="D15" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C15,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C15,User!$A:$A,0))</f>
         <v>org_user1_2</v>
       </c>
       <c r="E15" s="19" t="b">
@@ -12478,11 +12566,11 @@
         <v>0</v>
       </c>
       <c r="F15" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C15,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C15,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G15" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C15,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C15,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H15" s="6">
@@ -12564,7 +12652,7 @@
         <v>13</v>
       </c>
       <c r="D16" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C16,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C16,User!$A:$A,0))</f>
         <v>org_user1_3</v>
       </c>
       <c r="E16" s="19" t="b">
@@ -12572,11 +12660,11 @@
         <v>0</v>
       </c>
       <c r="F16" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C16,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C16,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G16" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C16,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C16,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H16" s="6">
@@ -12658,7 +12746,7 @@
         <v>14</v>
       </c>
       <c r="D17" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C17,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C17,User!$A:$A,0))</f>
         <v>org_user1_4</v>
       </c>
       <c r="E17" s="19" t="b">
@@ -12666,11 +12754,11 @@
         <v>0</v>
       </c>
       <c r="F17" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C17,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C17,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="G17" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C17,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C17,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H17" s="6">
@@ -12752,7 +12840,7 @@
         <v>16</v>
       </c>
       <c r="D18" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C18,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C18,User!$A:$A,0))</f>
         <v>org_user2_1</v>
       </c>
       <c r="E18" s="19" t="b">
@@ -12760,11 +12848,11 @@
         <v>0</v>
       </c>
       <c r="F18" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C18,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C18,User!$A:$A,0))</f>
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3</v>
       </c>
       <c r="G18" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C18,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C18,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H18" s="6" t="str">
@@ -12846,7 +12934,7 @@
         <v>18</v>
       </c>
       <c r="D19" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C19,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C19,User!$A:$A,0))</f>
         <v>org_user2_2</v>
       </c>
       <c r="E19" s="19" t="b">
@@ -12854,11 +12942,11 @@
         <v>0</v>
       </c>
       <c r="F19" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C19,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C19,User!$A:$A,0))</f>
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3</v>
       </c>
       <c r="G19" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C19,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C19,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H19" s="6" t="str">
@@ -12940,7 +13028,7 @@
         <v>19</v>
       </c>
       <c r="D20" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C20,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C20,User!$A:$A,0))</f>
         <v>org_user2_3</v>
       </c>
       <c r="E20" s="19" t="b">
@@ -12948,11 +13036,11 @@
         <v>0</v>
       </c>
       <c r="F20" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C20,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C20,User!$A:$A,0))</f>
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3</v>
       </c>
       <c r="G20" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C20,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C20,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H20" s="6" t="str">
@@ -13034,7 +13122,7 @@
         <v>20</v>
       </c>
       <c r="D21" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C21,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C21,User!$A:$A,0))</f>
         <v>org_user2_4</v>
       </c>
       <c r="E21" s="19" t="b">
@@ -13042,11 +13130,11 @@
         <v>0</v>
       </c>
       <c r="F21" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C21,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C21,User!$A:$A,0))</f>
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3</v>
       </c>
       <c r="G21" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C21,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C21,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H21" s="6" t="str">
@@ -13128,7 +13216,7 @@
         <v>22</v>
       </c>
       <c r="D22" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C22,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C22,User!$A:$A,0))</f>
         <v>org_user3_1</v>
       </c>
       <c r="E22" s="19" t="b">
@@ -13136,11 +13224,11 @@
         <v>0</v>
       </c>
       <c r="F22" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C22,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C22,User!$A:$A,0))</f>
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037</v>
       </c>
       <c r="G22" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C22,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C22,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H22" s="6" t="str">
@@ -13222,7 +13310,7 @@
         <v>24</v>
       </c>
       <c r="D23" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C23,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C23,User!$A:$A,0))</f>
         <v>org_user3_2</v>
       </c>
       <c r="E23" s="19" t="b">
@@ -13230,11 +13318,11 @@
         <v>0</v>
       </c>
       <c r="F23" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C23,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C23,User!$A:$A,0))</f>
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037</v>
       </c>
       <c r="G23" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C23,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C23,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H23" s="6" t="str">
@@ -13316,7 +13404,7 @@
         <v>25</v>
       </c>
       <c r="D24" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C24,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C24,User!$A:$A,0))</f>
         <v>org_user3_3</v>
       </c>
       <c r="E24" s="19" t="b">
@@ -13324,11 +13412,11 @@
         <v>0</v>
       </c>
       <c r="F24" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C24,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C24,User!$A:$A,0))</f>
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037</v>
       </c>
       <c r="G24" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C24,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C24,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H24" s="6" t="str">
@@ -13410,7 +13498,7 @@
         <v>26</v>
       </c>
       <c r="D25" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C25,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C25,User!$A:$A,0))</f>
         <v>org_user3_4</v>
       </c>
       <c r="E25" s="19" t="b">
@@ -13418,11 +13506,11 @@
         <v>0</v>
       </c>
       <c r="F25" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C25,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C25,User!$A:$A,0))</f>
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037</v>
       </c>
       <c r="G25" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C25,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C25,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H25" s="6" t="str">
@@ -13504,7 +13592,7 @@
         <v>28</v>
       </c>
       <c r="D26" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C26,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C26,User!$A:$A,0))</f>
         <v>org_user4_1</v>
       </c>
       <c r="E26" s="19" t="b">
@@ -13512,11 +13600,11 @@
         <v>0</v>
       </c>
       <c r="F26" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C26,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C26,User!$A:$A,0))</f>
         <v>0195d18c-1c92-d419-4c71-a570f428499b</v>
       </c>
       <c r="G26" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C26,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C26,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H26" s="6" t="str">
@@ -13598,7 +13686,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C27,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C27,User!$A:$A,0))</f>
         <v>org_user4_2</v>
       </c>
       <c r="E27" s="19" t="b">
@@ -13606,11 +13694,11 @@
         <v>0</v>
       </c>
       <c r="F27" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C27,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C27,User!$A:$A,0))</f>
         <v>0195d18c-1c92-d419-4c71-a570f428499b</v>
       </c>
       <c r="G27" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C27,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C27,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H27" s="6" t="str">
@@ -13692,7 +13780,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C28,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C28,User!$A:$A,0))</f>
         <v>org_user4_3</v>
       </c>
       <c r="E28" s="19" t="b">
@@ -13700,11 +13788,11 @@
         <v>0</v>
       </c>
       <c r="F28" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C28,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C28,User!$A:$A,0))</f>
         <v>0195d18c-1c92-d419-4c71-a570f428499b</v>
       </c>
       <c r="G28" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C28,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C28,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H28" s="6" t="str">
@@ -13786,7 +13874,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C29,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C29,User!$A:$A,0))</f>
         <v>org_user4_4</v>
       </c>
       <c r="E29" s="19" t="b">
@@ -13794,11 +13882,11 @@
         <v>0</v>
       </c>
       <c r="F29" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C29,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C29,User!$A:$A,0))</f>
         <v>0195d18c-1c92-d419-4c71-a570f428499b</v>
       </c>
       <c r="G29" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C29,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C29,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H29" s="6" t="str">
@@ -13880,7 +13968,7 @@
         <v>34</v>
       </c>
       <c r="D30" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C30,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C30,User!$A:$A,0))</f>
         <v>org_user5_1</v>
       </c>
       <c r="E30" s="19" t="b">
@@ -13888,11 +13976,11 @@
         <v>0</v>
       </c>
       <c r="F30" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C30,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C30,User!$A:$A,0))</f>
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0</v>
       </c>
       <c r="G30" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C30,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C30,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H30" s="6" t="str">
@@ -13974,7 +14062,7 @@
         <v>36</v>
       </c>
       <c r="D31" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C31,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C31,User!$A:$A,0))</f>
         <v>org_user5_2</v>
       </c>
       <c r="E31" s="19" t="b">
@@ -13982,11 +14070,11 @@
         <v>0</v>
       </c>
       <c r="F31" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C31,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C31,User!$A:$A,0))</f>
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0</v>
       </c>
       <c r="G31" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C31,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C31,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H31" s="6" t="str">
@@ -14068,7 +14156,7 @@
         <v>37</v>
       </c>
       <c r="D32" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C32,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C32,User!$A:$A,0))</f>
         <v>org_user5_3</v>
       </c>
       <c r="E32" s="19" t="b">
@@ -14076,11 +14164,11 @@
         <v>0</v>
       </c>
       <c r="F32" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C32,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C32,User!$A:$A,0))</f>
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0</v>
       </c>
       <c r="G32" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C32,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C32,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H32" s="6" t="str">
@@ -14162,7 +14250,7 @@
         <v>38</v>
       </c>
       <c r="D33" s="6" t="str">
-        <f>INDEX(User!$C:$C,MATCH($C33,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($C33,User!$A:$A,0))</f>
         <v>org_user5_4</v>
       </c>
       <c r="E33" s="19" t="b">
@@ -14170,11 +14258,11 @@
         <v>0</v>
       </c>
       <c r="F33" s="6" t="str">
-        <f>INDEX(User!$F:$F,MATCH($C33,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($C33,User!$A:$A,0))</f>
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0</v>
       </c>
       <c r="G33" s="6" t="b">
-        <f>INDEX(User!$L:$L,MATCH($C33,User!$A:$A,0))</f>
+        <f>INDEX(User!$M:$M,MATCH($C33,User!$A:$A,0))</f>
         <v>0</v>
       </c>
       <c r="H33" s="6" t="str">
@@ -21647,8 +21735,8 @@
         <v>44</v>
       </c>
       <c r="E2" t="str">
-        <f>VLOOKUP(D2,User!$A:$C,3,0)</f>
-        <v>org_admin1_1</v>
+        <f>VLOOKUP(D2,User!$A:$D,3,0)</f>
+        <v>org_admin1_1@org1_org</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -21669,8 +21757,8 @@
         <v>47</v>
       </c>
       <c r="E3" t="str">
-        <f>VLOOKUP(D3,User!$A:$C,3,0)</f>
-        <v>org_admin2_1</v>
+        <f>VLOOKUP(D3,User!$A:$D,3,0)</f>
+        <v>org_admin2_1@org2_org</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -21691,8 +21779,8 @@
         <v>50</v>
       </c>
       <c r="E4" t="str">
-        <f>VLOOKUP(D4,User!$A:$C,3,0)</f>
-        <v>org_admin3_1</v>
+        <f>VLOOKUP(D4,User!$A:$D,3,0)</f>
+        <v>org_admin3_1@org3_org</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -21713,8 +21801,8 @@
         <v>53</v>
       </c>
       <c r="E5" t="str">
-        <f>VLOOKUP(D5,User!$A:$C,3,0)</f>
-        <v>org_admin4_1</v>
+        <f>VLOOKUP(D5,User!$A:$D,3,0)</f>
+        <v>org_admin4_1@org4_org</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -21735,8 +21823,8 @@
         <v>56</v>
       </c>
       <c r="E6" t="str">
-        <f>VLOOKUP(D6,User!$A:$C,3,0)</f>
-        <v>org_admin5_1</v>
+        <f>VLOOKUP(D6,User!$A:$D,3,0)</f>
+        <v>org_admin5_1@org5_org</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -22747,7 +22835,7 @@
         <v>1</v>
       </c>
       <c r="Q2" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U2,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U2,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="R2" s="4" t="str">
@@ -22766,7 +22854,7 @@
         <v>10</v>
       </c>
       <c r="V2" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U2,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U2,User!$A:$A,0))</f>
         <v>org_user1_1</v>
       </c>
       <c r="W2" s="6" t="str">
@@ -22828,7 +22916,7 @@
         <v>1</v>
       </c>
       <c r="Q3" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U3,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U3,User!$A:$A,0))</f>
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3</v>
       </c>
       <c r="R3" s="4" t="str">
@@ -22847,7 +22935,7 @@
         <v>16</v>
       </c>
       <c r="V3" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U3,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U3,User!$A:$A,0))</f>
         <v>org_user2_1</v>
       </c>
       <c r="W3" s="6" t="str">
@@ -22909,7 +22997,7 @@
         <v>1</v>
       </c>
       <c r="Q4" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U4,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U4,User!$A:$A,0))</f>
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037</v>
       </c>
       <c r="R4" s="4" t="str">
@@ -22928,7 +23016,7 @@
         <v>22</v>
       </c>
       <c r="V4" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U4,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U4,User!$A:$A,0))</f>
         <v>org_user3_1</v>
       </c>
       <c r="W4" s="6" t="str">
@@ -22990,7 +23078,7 @@
         <v>1</v>
       </c>
       <c r="Q5" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U5,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U5,User!$A:$A,0))</f>
         <v>0195d18c-1c92-d419-4c71-a570f428499b</v>
       </c>
       <c r="R5" s="4" t="str">
@@ -23009,7 +23097,7 @@
         <v>28</v>
       </c>
       <c r="V5" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U5,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U5,User!$A:$A,0))</f>
         <v>org_user4_1</v>
       </c>
       <c r="W5" s="6" t="str">
@@ -23071,7 +23159,7 @@
         <v>1</v>
       </c>
       <c r="Q6" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U6,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U6,User!$A:$A,0))</f>
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0</v>
       </c>
       <c r="R6" s="4" t="str">
@@ -23090,7 +23178,7 @@
         <v>34</v>
       </c>
       <c r="V6" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U6,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U6,User!$A:$A,0))</f>
         <v>org_user5_1</v>
       </c>
       <c r="W6" s="6" t="str">
@@ -23152,7 +23240,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U7,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U7,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="R7" s="4" t="str">
@@ -23171,7 +23259,7 @@
         <v>10</v>
       </c>
       <c r="V7" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U7,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U7,User!$A:$A,0))</f>
         <v>org_user1_1</v>
       </c>
       <c r="W7" s="6" t="str">
@@ -23233,7 +23321,7 @@
         <v>1</v>
       </c>
       <c r="Q8" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U8,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U8,User!$A:$A,0))</f>
         <v>0195d18c-1c92-0ed4-2e94-b4f66d82baf3</v>
       </c>
       <c r="R8" s="4" t="str">
@@ -23252,7 +23340,7 @@
         <v>16</v>
       </c>
       <c r="V8" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U8,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U8,User!$A:$A,0))</f>
         <v>org_user2_1</v>
       </c>
       <c r="W8" s="6" t="str">
@@ -23314,7 +23402,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U9,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U9,User!$A:$A,0))</f>
         <v>0195d18c-1c92-52b3-93e0-43dc1f2aa037</v>
       </c>
       <c r="R9" s="4" t="str">
@@ -23333,7 +23421,7 @@
         <v>22</v>
       </c>
       <c r="V9" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U9,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U9,User!$A:$A,0))</f>
         <v>org_user3_1</v>
       </c>
       <c r="W9" s="6" t="str">
@@ -23395,7 +23483,7 @@
         <v>1</v>
       </c>
       <c r="Q10" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U10,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U10,User!$A:$A,0))</f>
         <v>0195d18c-1c92-d419-4c71-a570f428499b</v>
       </c>
       <c r="R10" s="4" t="str">
@@ -23414,7 +23502,7 @@
         <v>28</v>
       </c>
       <c r="V10" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U10,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U10,User!$A:$A,0))</f>
         <v>org_user4_1</v>
       </c>
       <c r="W10" s="6" t="str">
@@ -23476,7 +23564,7 @@
         <v>1</v>
       </c>
       <c r="Q11" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($U11,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($U11,User!$A:$A,0))</f>
         <v>0195d18c-1c93-02a2-6920-7e4dbfb73ce0</v>
       </c>
       <c r="R11" s="4" t="str">
@@ -23495,7 +23583,7 @@
         <v>34</v>
       </c>
       <c r="V11" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($U11,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($U11,User!$A:$A,0))</f>
         <v>org_user5_1</v>
       </c>
       <c r="W11" s="6" t="str">
@@ -23626,7 +23714,7 @@
         <v>data_collection1</v>
       </c>
       <c r="M2" s="4" t="str">
-        <f>INDEX(User!$F:$F,MATCH($O2,User!$A:$A,0))</f>
+        <f>INDEX(User!$G:$G,MATCH($O2,User!$A:$A,0))</f>
         <v>018d074d-ea0c-e942-07db-a3cc0ba1d653</v>
       </c>
       <c r="N2" s="4" t="str">
@@ -23637,7 +23725,7 @@
         <v>10</v>
       </c>
       <c r="P2" s="4" t="str">
-        <f>INDEX(User!$C:$C,MATCH($O2,User!$A:$A,0))</f>
+        <f>INDEX(User!$D:$D,MATCH($O2,User!$A:$A,0))</f>
         <v>org_user1_1</v>
       </c>
     </row>
@@ -25316,1322 +25404,1411 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="36" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.33203125" customWidth="1"/>
+    <col min="3" max="3" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.77734375" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>874</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>803</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>804</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>805</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>806</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>807</v>
       </c>
-      <c r="L1" s="17" t="s">
+      <c r="M1" s="17" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>873</v>
       </c>
       <c r="B2" t="s">
         <v>757</v>
       </c>
-      <c r="C2" t="str">
-        <f>LEFT(B2,FIND("@",B2)-1)</f>
+      <c r="C2" t="s">
+        <v>757</v>
+      </c>
+      <c r="D2" t="str">
+        <f>LEFT(C2,FIND("@",C2)-1)</f>
         <v>root1_1</v>
       </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
         <v>274</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F2,Organization!$A:$A,0))</f>
+      <c r="H2" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G2,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
-      <c r="H2" s="18" t="b">
-        <f>ISNUMBER(SEARCH("ROOT", E2))</f>
-        <v>1</v>
-      </c>
       <c r="I2" s="18" t="b">
-        <f>ISNUMBER(SEARCH("APP_ADMIN", $E2))</f>
-        <v>0</v>
+        <f>ISNUMBER(SEARCH("ROOT", F2))</f>
+        <v>1</v>
       </c>
       <c r="J2" s="18" t="b">
-        <f>ISNUMBER(SEARCH("METADATA_ADMIN", $E2))</f>
+        <f>ISNUMBER(SEARCH("APP_ADMIN", $F2))</f>
         <v>0</v>
       </c>
       <c r="K2" s="18" t="b">
-        <f>ISNUMBER(SEARCH("ORG_USER", $E2))</f>
-        <v>0</v>
-      </c>
-      <c r="L2" s="6" t="b">
-        <f>OR($H2,$I2)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+        <f>ISNUMBER(SEARCH("METADATA_ADMIN", $F2))</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="18" t="b">
+        <f>ISNUMBER(SEARCH("ORG_USER", $F2))</f>
+        <v>0</v>
+      </c>
+      <c r="M2" s="6" t="b">
+        <f>OR($I2,$J2)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>192</v>
       </c>
       <c r="B3" t="s">
         <v>758</v>
       </c>
-      <c r="C3" t="str">
-        <f t="shared" ref="C3:C29" si="0">LEFT(B3,FIND("@",B3)-1)</f>
+      <c r="C3" t="s">
+        <v>758</v>
+      </c>
+      <c r="D3" t="str">
+        <f t="shared" ref="D3:D29" si="0">LEFT(C3,FIND("@",C3)-1)</f>
         <v>app_admin1_1</v>
       </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
         <v>275</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F3,Organization!$A:$A,0))</f>
+      <c r="H3" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G3,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
-      <c r="H3" s="18" t="b">
-        <f t="shared" ref="H3:H29" si="1">ISNUMBER(SEARCH("ROOT", E3))</f>
-        <v>0</v>
-      </c>
       <c r="I3" s="18" t="b">
-        <f t="shared" ref="I3:I29" si="2">ISNUMBER(SEARCH("APP_ADMIN", $E3))</f>
-        <v>1</v>
+        <f t="shared" ref="I3:I29" si="1">ISNUMBER(SEARCH("ROOT", F3))</f>
+        <v>0</v>
       </c>
       <c r="J3" s="18" t="b">
-        <f t="shared" ref="J3:J29" si="3">ISNUMBER(SEARCH("METADATA_ADMIN", $E3))</f>
-        <v>0</v>
+        <f t="shared" ref="J3:J29" si="2">ISNUMBER(SEARCH("APP_ADMIN", $F3))</f>
+        <v>1</v>
       </c>
       <c r="K3" s="18" t="b">
-        <f t="shared" ref="K3:K29" si="4">ISNUMBER(SEARCH("ORG_USER", $E3))</f>
-        <v>0</v>
-      </c>
-      <c r="L3" s="6" t="b">
-        <f t="shared" ref="L3:L29" si="5">OR($H3,$I3)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+        <f t="shared" ref="K3:K29" si="3">ISNUMBER(SEARCH("METADATA_ADMIN", $F3))</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="18" t="b">
+        <f t="shared" ref="L3:L29" si="4">ISNUMBER(SEARCH("ORG_USER", $F3))</f>
+        <v>0</v>
+      </c>
+      <c r="M3" s="6" t="b">
+        <f t="shared" ref="M3:M29" si="5">OR($I3,$J3)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>193</v>
       </c>
       <c r="B4" s="20" t="s">
         <v>759</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C4" s="20" t="s">
+        <v>759</v>
+      </c>
+      <c r="D4" t="str">
         <f t="shared" si="0"/>
         <v>refdata_admin1_1</v>
       </c>
-      <c r="D4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
         <v>304</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F4,Organization!$A:$A,0))</f>
+      <c r="H4" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G4,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
-      <c r="H4" s="18" t="b">
+      <c r="I4" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I4" s="18" t="b">
+      <c r="J4" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J4" s="18" t="b">
+      <c r="K4" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K4" s="18" t="b">
+      <c r="L4" s="18" t="b">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="L4" s="6" t="b">
+      <c r="M4" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>44</v>
       </c>
       <c r="B5" t="s">
         <v>760</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C5" t="s">
+        <v>760</v>
+      </c>
+      <c r="D5" t="str">
         <f t="shared" si="0"/>
         <v>org_admin1_1</v>
       </c>
-      <c r="D5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
         <v>276</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F5,Organization!$A:$A,0))</f>
+      <c r="H5" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G5,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
-      <c r="H5" s="18" t="b">
+      <c r="I5" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I5" s="18" t="b">
+      <c r="J5" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J5" s="18" t="b">
+      <c r="K5" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K5" s="18" t="b">
+      <c r="L5" s="18" t="b">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="L5" s="6" t="b">
+      <c r="M5" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>47</v>
       </c>
       <c r="B6" t="s">
         <v>761</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C6" t="s">
+        <v>761</v>
+      </c>
+      <c r="D6" t="str">
         <f t="shared" si="0"/>
         <v>org_admin2_1</v>
       </c>
-      <c r="D6" t="b">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
         <v>276</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F6,Organization!$A:$A,0))</f>
+      <c r="H6" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G6,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
-      <c r="H6" s="18" t="b">
+      <c r="I6" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I6" s="18" t="b">
+      <c r="J6" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J6" s="18" t="b">
+      <c r="K6" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K6" s="18" t="b">
+      <c r="L6" s="18" t="b">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="L6" s="6" t="b">
+      <c r="M6" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>50</v>
       </c>
       <c r="B7" t="s">
         <v>762</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C7" t="s">
+        <v>762</v>
+      </c>
+      <c r="D7" t="str">
         <f t="shared" si="0"/>
         <v>org_admin3_1</v>
       </c>
-      <c r="D7" t="b">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
         <v>276</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>49</v>
       </c>
-      <c r="G7" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F7,Organization!$A:$A,0))</f>
+      <c r="H7" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G7,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
-      <c r="H7" s="18" t="b">
+      <c r="I7" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I7" s="18" t="b">
+      <c r="J7" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J7" s="18" t="b">
+      <c r="K7" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K7" s="18" t="b">
+      <c r="L7" s="18" t="b">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="L7" s="6" t="b">
+      <c r="M7" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>53</v>
       </c>
       <c r="B8" t="s">
         <v>763</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C8" t="s">
+        <v>763</v>
+      </c>
+      <c r="D8" t="str">
         <f t="shared" si="0"/>
         <v>org_admin4_1</v>
       </c>
-      <c r="D8" t="b">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
         <v>276</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>52</v>
       </c>
-      <c r="G8" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F8,Organization!$A:$A,0))</f>
+      <c r="H8" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G8,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
-      <c r="H8" s="18" t="b">
+      <c r="I8" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I8" s="18" t="b">
+      <c r="J8" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J8" s="18" t="b">
+      <c r="K8" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K8" s="18" t="b">
+      <c r="L8" s="18" t="b">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="L8" s="6" t="b">
+      <c r="M8" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>56</v>
       </c>
       <c r="B9" t="s">
         <v>764</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C9" t="s">
+        <v>764</v>
+      </c>
+      <c r="D9" t="str">
         <f t="shared" si="0"/>
         <v>org_admin5_1</v>
       </c>
-      <c r="D9" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
         <v>276</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F9,Organization!$A:$A,0))</f>
+      <c r="H9" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G9,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
-      <c r="H9" s="18" t="b">
+      <c r="I9" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I9" s="18" t="b">
+      <c r="J9" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J9" s="18" t="b">
+      <c r="K9" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K9" s="18" t="b">
+      <c r="L9" s="18" t="b">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="L9" s="6" t="b">
+      <c r="M9" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10" t="s">
         <v>765</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C10" t="s">
+        <v>765</v>
+      </c>
+      <c r="D10" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_1</v>
       </c>
-      <c r="D10" t="b">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
         <v>277</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F10,Organization!$A:$A,0))</f>
+      <c r="H10" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G10,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
-      <c r="H10" s="18" t="b">
+      <c r="I10" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I10" s="18" t="b">
+      <c r="J10" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J10" s="18" t="b">
+      <c r="K10" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K10" s="18" t="b">
+      <c r="L10" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L10" s="6" t="b">
+      <c r="M10" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
       <c r="B11" t="s">
         <v>766</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C11" t="s">
+        <v>766</v>
+      </c>
+      <c r="D11" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_2</v>
       </c>
-      <c r="D11" t="b">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
         <v>277</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>43</v>
       </c>
-      <c r="G11" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F11,Organization!$A:$A,0))</f>
+      <c r="H11" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G11,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
-      <c r="H11" s="18" t="b">
+      <c r="I11" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I11" s="18" t="b">
+      <c r="J11" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J11" s="18" t="b">
+      <c r="K11" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K11" s="18" t="b">
+      <c r="L11" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L11" s="6" t="b">
+      <c r="M11" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" t="s">
         <v>767</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C12" t="s">
+        <v>767</v>
+      </c>
+      <c r="D12" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_3</v>
       </c>
-      <c r="D12" t="b">
-        <v>1</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
         <v>277</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F12,Organization!$A:$A,0))</f>
+      <c r="H12" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G12,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
-      <c r="H12" s="18" t="b">
+      <c r="I12" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I12" s="18" t="b">
+      <c r="J12" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J12" s="18" t="b">
+      <c r="K12" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K12" s="18" t="b">
+      <c r="L12" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L12" s="6" t="b">
+      <c r="M12" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>14</v>
       </c>
       <c r="B13" t="s">
         <v>768</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C13" t="s">
+        <v>768</v>
+      </c>
+      <c r="D13" t="str">
         <f t="shared" si="0"/>
         <v>org_user1_4</v>
       </c>
-      <c r="D13" t="b">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
         <v>277</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>43</v>
       </c>
-      <c r="G13" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F13,Organization!$A:$A,0))</f>
+      <c r="H13" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G13,Organization!$A:$A,0))</f>
         <v>org1</v>
       </c>
-      <c r="H13" s="18" t="b">
+      <c r="I13" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I13" s="18" t="b">
+      <c r="J13" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J13" s="18" t="b">
+      <c r="K13" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K13" s="18" t="b">
+      <c r="L13" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L13" s="6" t="b">
+      <c r="M13" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>16</v>
       </c>
       <c r="B14" t="s">
         <v>769</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C14" t="s">
+        <v>769</v>
+      </c>
+      <c r="D14" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_1</v>
       </c>
-      <c r="D14" t="b">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
         <v>277</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>46</v>
       </c>
-      <c r="G14" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F14,Organization!$A:$A,0))</f>
+      <c r="H14" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G14,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
-      <c r="H14" s="18" t="b">
+      <c r="I14" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I14" s="18" t="b">
+      <c r="J14" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J14" s="18" t="b">
+      <c r="K14" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K14" s="18" t="b">
+      <c r="L14" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L14" s="6" t="b">
+      <c r="M14" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>18</v>
       </c>
       <c r="B15" t="s">
         <v>770</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C15" t="s">
+        <v>770</v>
+      </c>
+      <c r="D15" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_2</v>
       </c>
-      <c r="D15" t="b">
-        <v>1</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
         <v>277</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F15,Organization!$A:$A,0))</f>
+      <c r="H15" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G15,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
-      <c r="H15" s="18" t="b">
+      <c r="I15" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I15" s="18" t="b">
+      <c r="J15" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J15" s="18" t="b">
+      <c r="K15" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K15" s="18" t="b">
+      <c r="L15" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L15" s="6" t="b">
+      <c r="M15" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>19</v>
       </c>
       <c r="B16" t="s">
         <v>771</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C16" t="s">
+        <v>771</v>
+      </c>
+      <c r="D16" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_3</v>
       </c>
-      <c r="D16" t="b">
-        <v>1</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
         <v>277</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>46</v>
       </c>
-      <c r="G16" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F16,Organization!$A:$A,0))</f>
+      <c r="H16" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G16,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
-      <c r="H16" s="18" t="b">
+      <c r="I16" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I16" s="18" t="b">
+      <c r="J16" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J16" s="18" t="b">
+      <c r="K16" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K16" s="18" t="b">
+      <c r="L16" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L16" s="6" t="b">
+      <c r="M16" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>20</v>
       </c>
       <c r="B17" t="s">
         <v>772</v>
       </c>
-      <c r="C17" t="str">
+      <c r="C17" t="s">
+        <v>772</v>
+      </c>
+      <c r="D17" t="str">
         <f t="shared" si="0"/>
         <v>org_user2_4</v>
       </c>
-      <c r="D17" t="b">
-        <v>1</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
         <v>277</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>46</v>
       </c>
-      <c r="G17" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F17,Organization!$A:$A,0))</f>
+      <c r="H17" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G17,Organization!$A:$A,0))</f>
         <v>org2</v>
       </c>
-      <c r="H17" s="18" t="b">
+      <c r="I17" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I17" s="18" t="b">
+      <c r="J17" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J17" s="18" t="b">
+      <c r="K17" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K17" s="18" t="b">
+      <c r="L17" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L17" s="6" t="b">
+      <c r="M17" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>22</v>
       </c>
       <c r="B18" t="s">
         <v>773</v>
       </c>
-      <c r="C18" t="str">
+      <c r="C18" t="s">
+        <v>773</v>
+      </c>
+      <c r="D18" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_1</v>
       </c>
-      <c r="D18" t="b">
-        <v>1</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
         <v>277</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>49</v>
       </c>
-      <c r="G18" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F18,Organization!$A:$A,0))</f>
+      <c r="H18" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G18,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
-      <c r="H18" s="18" t="b">
+      <c r="I18" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I18" s="18" t="b">
+      <c r="J18" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J18" s="18" t="b">
+      <c r="K18" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K18" s="18" t="b">
+      <c r="L18" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L18" s="6" t="b">
+      <c r="M18" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>24</v>
       </c>
       <c r="B19" t="s">
         <v>774</v>
       </c>
-      <c r="C19" t="str">
+      <c r="C19" t="s">
+        <v>774</v>
+      </c>
+      <c r="D19" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_2</v>
       </c>
-      <c r="D19" t="b">
-        <v>1</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
         <v>277</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>49</v>
       </c>
-      <c r="G19" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F19,Organization!$A:$A,0))</f>
+      <c r="H19" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G19,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
-      <c r="H19" s="18" t="b">
+      <c r="I19" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I19" s="18" t="b">
+      <c r="J19" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J19" s="18" t="b">
+      <c r="K19" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K19" s="18" t="b">
+      <c r="L19" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L19" s="6" t="b">
+      <c r="M19" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>25</v>
       </c>
       <c r="B20" t="s">
         <v>775</v>
       </c>
-      <c r="C20" t="str">
+      <c r="C20" t="s">
+        <v>775</v>
+      </c>
+      <c r="D20" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_3</v>
       </c>
-      <c r="D20" t="b">
-        <v>1</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" t="s">
         <v>277</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>49</v>
       </c>
-      <c r="G20" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F20,Organization!$A:$A,0))</f>
+      <c r="H20" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G20,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
-      <c r="H20" s="18" t="b">
+      <c r="I20" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I20" s="18" t="b">
+      <c r="J20" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J20" s="18" t="b">
+      <c r="K20" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K20" s="18" t="b">
+      <c r="L20" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L20" s="6" t="b">
+      <c r="M20" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>26</v>
       </c>
       <c r="B21" t="s">
         <v>776</v>
       </c>
-      <c r="C21" t="str">
+      <c r="C21" t="s">
+        <v>776</v>
+      </c>
+      <c r="D21" t="str">
         <f t="shared" si="0"/>
         <v>org_user3_4</v>
       </c>
-      <c r="D21" t="b">
-        <v>1</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
         <v>277</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>49</v>
       </c>
-      <c r="G21" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F21,Organization!$A:$A,0))</f>
+      <c r="H21" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G21,Organization!$A:$A,0))</f>
         <v>org3</v>
       </c>
-      <c r="H21" s="18" t="b">
+      <c r="I21" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I21" s="18" t="b">
+      <c r="J21" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J21" s="18" t="b">
+      <c r="K21" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K21" s="18" t="b">
+      <c r="L21" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L21" s="6" t="b">
+      <c r="M21" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>28</v>
       </c>
       <c r="B22" t="s">
         <v>777</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C22" t="s">
+        <v>777</v>
+      </c>
+      <c r="D22" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_1</v>
       </c>
-      <c r="D22" t="b">
-        <v>1</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
         <v>277</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>52</v>
       </c>
-      <c r="G22" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F22,Organization!$A:$A,0))</f>
+      <c r="H22" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G22,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
-      <c r="H22" s="18" t="b">
+      <c r="I22" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I22" s="18" t="b">
+      <c r="J22" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J22" s="18" t="b">
+      <c r="K22" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K22" s="18" t="b">
+      <c r="L22" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L22" s="6" t="b">
+      <c r="M22" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>30</v>
       </c>
       <c r="B23" t="s">
         <v>778</v>
       </c>
-      <c r="C23" t="str">
+      <c r="C23" t="s">
+        <v>778</v>
+      </c>
+      <c r="D23" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_2</v>
       </c>
-      <c r="D23" t="b">
-        <v>1</v>
-      </c>
-      <c r="E23" t="s">
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" t="s">
         <v>277</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>52</v>
       </c>
-      <c r="G23" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F23,Organization!$A:$A,0))</f>
+      <c r="H23" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G23,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
-      <c r="H23" s="18" t="b">
+      <c r="I23" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I23" s="18" t="b">
+      <c r="J23" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J23" s="18" t="b">
+      <c r="K23" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K23" s="18" t="b">
+      <c r="L23" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L23" s="6" t="b">
+      <c r="M23" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>31</v>
       </c>
       <c r="B24" t="s">
         <v>779</v>
       </c>
-      <c r="C24" t="str">
+      <c r="C24" t="s">
+        <v>779</v>
+      </c>
+      <c r="D24" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_3</v>
       </c>
-      <c r="D24" t="b">
-        <v>1</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" t="s">
         <v>277</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>52</v>
       </c>
-      <c r="G24" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F24,Organization!$A:$A,0))</f>
+      <c r="H24" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G24,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
-      <c r="H24" s="18" t="b">
+      <c r="I24" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I24" s="18" t="b">
+      <c r="J24" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J24" s="18" t="b">
+      <c r="K24" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K24" s="18" t="b">
+      <c r="L24" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L24" s="6" t="b">
+      <c r="M24" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>32</v>
       </c>
       <c r="B25" t="s">
         <v>780</v>
       </c>
-      <c r="C25" t="str">
+      <c r="C25" t="s">
+        <v>780</v>
+      </c>
+      <c r="D25" t="str">
         <f t="shared" si="0"/>
         <v>org_user4_4</v>
       </c>
-      <c r="D25" t="b">
-        <v>1</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="E25" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" t="s">
         <v>277</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>52</v>
       </c>
-      <c r="G25" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F25,Organization!$A:$A,0))</f>
+      <c r="H25" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G25,Organization!$A:$A,0))</f>
         <v>org4</v>
       </c>
-      <c r="H25" s="18" t="b">
+      <c r="I25" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I25" s="18" t="b">
+      <c r="J25" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J25" s="18" t="b">
+      <c r="K25" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K25" s="18" t="b">
+      <c r="L25" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L25" s="6" t="b">
+      <c r="M25" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>34</v>
       </c>
       <c r="B26" t="s">
         <v>781</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C26" t="s">
+        <v>781</v>
+      </c>
+      <c r="D26" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_1</v>
       </c>
-      <c r="D26" t="b">
-        <v>1</v>
-      </c>
-      <c r="E26" t="s">
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
         <v>277</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>55</v>
       </c>
-      <c r="G26" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F26,Organization!$A:$A,0))</f>
+      <c r="H26" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G26,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
-      <c r="H26" s="18" t="b">
+      <c r="I26" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I26" s="18" t="b">
+      <c r="J26" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J26" s="18" t="b">
+      <c r="K26" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K26" s="18" t="b">
+      <c r="L26" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L26" s="6" t="b">
+      <c r="M26" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>36</v>
       </c>
       <c r="B27" t="s">
         <v>782</v>
       </c>
-      <c r="C27" t="str">
+      <c r="C27" t="s">
+        <v>782</v>
+      </c>
+      <c r="D27" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_2</v>
       </c>
-      <c r="D27" t="b">
-        <v>1</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="E27" t="b">
+        <v>1</v>
+      </c>
+      <c r="F27" t="s">
         <v>277</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>55</v>
       </c>
-      <c r="G27" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F27,Organization!$A:$A,0))</f>
+      <c r="H27" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G27,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
-      <c r="H27" s="18" t="b">
+      <c r="I27" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I27" s="18" t="b">
+      <c r="J27" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J27" s="18" t="b">
+      <c r="K27" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K27" s="18" t="b">
+      <c r="L27" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L27" s="6" t="b">
+      <c r="M27" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
       <c r="B28" t="s">
         <v>783</v>
       </c>
-      <c r="C28" t="str">
+      <c r="C28" t="s">
+        <v>783</v>
+      </c>
+      <c r="D28" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_3</v>
       </c>
-      <c r="D28" t="b">
-        <v>1</v>
-      </c>
-      <c r="E28" t="s">
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
         <v>277</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>55</v>
       </c>
-      <c r="G28" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F28,Organization!$A:$A,0))</f>
+      <c r="H28" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G28,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
-      <c r="H28" s="18" t="b">
+      <c r="I28" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I28" s="18" t="b">
+      <c r="J28" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J28" s="18" t="b">
+      <c r="K28" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K28" s="18" t="b">
+      <c r="L28" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L28" s="6" t="b">
+      <c r="M28" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>38</v>
       </c>
       <c r="B29" t="s">
         <v>784</v>
       </c>
-      <c r="C29" t="str">
+      <c r="C29" t="s">
+        <v>784</v>
+      </c>
+      <c r="D29" t="str">
         <f t="shared" si="0"/>
         <v>org_user5_4</v>
       </c>
-      <c r="D29" t="b">
-        <v>1</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="E29" t="b">
+        <v>1</v>
+      </c>
+      <c r="F29" t="s">
         <v>277</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>55</v>
       </c>
-      <c r="G29" s="18" t="str">
-        <f>INDEX(Organization!$B:$B,MATCH($F29,Organization!$A:$A,0))</f>
+      <c r="H29" s="18" t="str">
+        <f>INDEX(Organization!$B:$B,MATCH($G29,Organization!$A:$A,0))</f>
         <v>org5</v>
       </c>
-      <c r="H29" s="18" t="b">
+      <c r="I29" s="18" t="b">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I29" s="18" t="b">
+      <c r="J29" s="18" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J29" s="18" t="b">
+      <c r="K29" s="18" t="b">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K29" s="18" t="b">
+      <c r="L29" s="18" t="b">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="L29" s="6" t="b">
+      <c r="M29" s="6" t="b">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B4" r:id="rId1" display="refdata_admin1_1@org1.org" xr:uid="{6720259D-8B8B-404B-BBFC-255A858BC201}"/>
+    <hyperlink ref="C4" r:id="rId1" display="refdata_admin1_1@org1.org" xr:uid="{6720259D-8B8B-404B-BBFC-255A858BC201}"/>
+    <hyperlink ref="B4" r:id="rId2" display="refdata_admin1_1@org1.org" xr:uid="{20728C37-5C65-48C8-8BFF-B78EF176652E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: commondb UserManager create_root_user_from_claims updated refactor: removed root user id from toml
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F5C3440-E169-49AB-B04F-4AB419B33125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B50F3BB1-41BD-43FD-8DD5-18F1B5FB645A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3552" yWindow="3552" windowWidth="30960" windowHeight="12120" tabRatio="913" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4248" yWindow="4248" windowWidth="30960" windowHeight="12120" tabRatio="913" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="902">
   <si>
     <t>id</t>
   </si>
@@ -2380,9 +2380,6 @@
     <t>to_region_name</t>
   </si>
   <si>
-    <t>root1_1@org1_org</t>
-  </si>
-  <si>
     <t>app_admin1_1@org1_org</t>
   </si>
   <si>
@@ -2747,6 +2744,90 @@
   </si>
   <si>
     <t>["CASEDB_ROOT"]</t>
+  </si>
+  <si>
+    <t>root1_1@org1.org</t>
+  </si>
+  <si>
+    <t>app_admin1_1@org1.org</t>
+  </si>
+  <si>
+    <t>refdata_admin1_1@org1.org</t>
+  </si>
+  <si>
+    <t>org_admin1_1@org1.org</t>
+  </si>
+  <si>
+    <t>org_admin2_1@org2.org</t>
+  </si>
+  <si>
+    <t>org_admin3_1@org3.org</t>
+  </si>
+  <si>
+    <t>org_admin4_1@org4.org</t>
+  </si>
+  <si>
+    <t>org_admin5_1@org5.org</t>
+  </si>
+  <si>
+    <t>org_user1_1@org1.org</t>
+  </si>
+  <si>
+    <t>org_user1_2@org1.org</t>
+  </si>
+  <si>
+    <t>org_user1_3@org1.org</t>
+  </si>
+  <si>
+    <t>org_user1_4@org1.org</t>
+  </si>
+  <si>
+    <t>org_user2_1@org2.org</t>
+  </si>
+  <si>
+    <t>org_user2_2@org2.org</t>
+  </si>
+  <si>
+    <t>org_user2_3@org2.org</t>
+  </si>
+  <si>
+    <t>org_user2_4@org2.org</t>
+  </si>
+  <si>
+    <t>org_user3_1@org3.org</t>
+  </si>
+  <si>
+    <t>org_user3_2@org3.org</t>
+  </si>
+  <si>
+    <t>org_user3_3@org3.org</t>
+  </si>
+  <si>
+    <t>org_user3_4@org3.org</t>
+  </si>
+  <si>
+    <t>org_user4_1@org4.org</t>
+  </si>
+  <si>
+    <t>org_user4_2@org4.org</t>
+  </si>
+  <si>
+    <t>org_user4_3@org4.org</t>
+  </si>
+  <si>
+    <t>org_user4_4@org4.org</t>
+  </si>
+  <si>
+    <t>org_user5_1@org5.org</t>
+  </si>
+  <si>
+    <t>org_user5_2@org5.org</t>
+  </si>
+  <si>
+    <t>org_user5_3@org5.org</t>
+  </si>
+  <si>
+    <t>org_user5_4@org5.org</t>
   </si>
 </sst>
 </file>
@@ -3550,7 +3631,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>190</v>
@@ -3585,10 +3666,10 @@
         <v>217</v>
       </c>
       <c r="B2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="C2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="D2" s="6" t="str">
         <f>LEFT($C2,LEN($C2)-9)</f>
@@ -3601,10 +3682,10 @@
         <v>45743.390918726589</v>
       </c>
       <c r="G2" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="H2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="I2" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($H2,User!$A:$A,0))</f>
@@ -3623,10 +3704,10 @@
         <v>219</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="D3" s="6" t="str">
         <f t="shared" ref="D3:D28" si="0">LEFT($C3,LEN($C3)-9)</f>
@@ -3639,7 +3720,7 @@
         <v>45743.390918741461</v>
       </c>
       <c r="G3" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="H3" t="s">
         <v>192</v>
@@ -3661,10 +3742,10 @@
         <v>221</v>
       </c>
       <c r="B4" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="C4" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D4" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3677,7 +3758,7 @@
         <v>45743.390918746562</v>
       </c>
       <c r="G4" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H4" t="s">
         <v>192</v>
@@ -3699,10 +3780,10 @@
         <v>223</v>
       </c>
       <c r="B5" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="C5" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="D5" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3715,7 +3796,7 @@
         <v>45743.390918763551</v>
       </c>
       <c r="G5" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H5" t="s">
         <v>192</v>
@@ -3737,10 +3818,10 @@
         <v>225</v>
       </c>
       <c r="B6" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C6" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="D6" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3753,7 +3834,7 @@
         <v>45743.390918772537</v>
       </c>
       <c r="G6" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H6" t="s">
         <v>192</v>
@@ -3775,10 +3856,10 @@
         <v>227</v>
       </c>
       <c r="B7" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C7" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="D7" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3791,7 +3872,7 @@
         <v>45743.390918781181</v>
       </c>
       <c r="G7" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H7" t="s">
         <v>192</v>
@@ -3813,10 +3894,10 @@
         <v>229</v>
       </c>
       <c r="B8" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="C8" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D8" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3829,7 +3910,7 @@
         <v>45743.3909187889</v>
       </c>
       <c r="G8" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H8" t="s">
         <v>192</v>
@@ -3851,10 +3932,10 @@
         <v>231</v>
       </c>
       <c r="B9" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C9" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D9" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3867,7 +3948,7 @@
         <v>45743.390918796598</v>
       </c>
       <c r="G9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H9" t="s">
         <v>192</v>
@@ -3889,10 +3970,10 @@
         <v>233</v>
       </c>
       <c r="B10" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="C10" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="D10" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3905,7 +3986,7 @@
         <v>45743.390918801953</v>
       </c>
       <c r="G10" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H10" t="s">
         <v>192</v>
@@ -3927,10 +4008,10 @@
         <v>235</v>
       </c>
       <c r="B11" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="C11" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D11" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3943,7 +4024,7 @@
         <v>45743.390918807163</v>
       </c>
       <c r="G11" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H11" t="s">
         <v>192</v>
@@ -3965,10 +4046,10 @@
         <v>237</v>
       </c>
       <c r="B12" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="C12" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="D12" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3981,7 +4062,7 @@
         <v>45743.3909188123</v>
       </c>
       <c r="G12" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H12" t="s">
         <v>192</v>
@@ -4003,10 +4084,10 @@
         <v>239</v>
       </c>
       <c r="B13" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="C13" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="D13" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4019,7 +4100,7 @@
         <v>45743.390918817633</v>
       </c>
       <c r="G13" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H13" t="s">
         <v>192</v>
@@ -4041,10 +4122,10 @@
         <v>241</v>
       </c>
       <c r="B14" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="C14" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D14" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4057,7 +4138,7 @@
         <v>45743.390918822908</v>
       </c>
       <c r="G14" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H14" t="s">
         <v>192</v>
@@ -4079,10 +4160,10 @@
         <v>243</v>
       </c>
       <c r="B15" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="C15" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="D15" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4095,7 +4176,7 @@
         <v>45743.390918828743</v>
       </c>
       <c r="G15" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H15" t="s">
         <v>192</v>
@@ -4117,10 +4198,10 @@
         <v>245</v>
       </c>
       <c r="B16" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C16" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="D16" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4133,7 +4214,7 @@
         <v>45743.390918834302</v>
       </c>
       <c r="G16" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H16" t="s">
         <v>192</v>
@@ -4155,10 +4236,10 @@
         <v>247</v>
       </c>
       <c r="B17" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C17" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="D17" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4171,7 +4252,7 @@
         <v>45743.390918839839</v>
       </c>
       <c r="G17" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H17" t="s">
         <v>192</v>
@@ -4193,10 +4274,10 @@
         <v>249</v>
       </c>
       <c r="B18" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="C18" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="D18" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4209,7 +4290,7 @@
         <v>45743.390918845187</v>
       </c>
       <c r="G18" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H18" t="s">
         <v>192</v>
@@ -4231,10 +4312,10 @@
         <v>251</v>
       </c>
       <c r="B19" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C19" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D19" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4247,7 +4328,7 @@
         <v>45743.390918851088</v>
       </c>
       <c r="G19" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H19" t="s">
         <v>192</v>
@@ -4269,10 +4350,10 @@
         <v>253</v>
       </c>
       <c r="B20" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C20" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="D20" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4285,7 +4366,7 @@
         <v>45743.39091885696</v>
       </c>
       <c r="G20" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H20" t="s">
         <v>192</v>
@@ -4307,10 +4388,10 @@
         <v>255</v>
       </c>
       <c r="B21" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="C21" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="D21" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4323,7 +4404,7 @@
         <v>45743.390918862962</v>
       </c>
       <c r="G21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H21" t="s">
         <v>192</v>
@@ -4345,10 +4426,10 @@
         <v>257</v>
       </c>
       <c r="B22" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="C22" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D22" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4361,7 +4442,7 @@
         <v>45743.390918868739</v>
       </c>
       <c r="G22" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H22" t="s">
         <v>192</v>
@@ -4383,10 +4464,10 @@
         <v>259</v>
       </c>
       <c r="B23" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="C23" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="D23" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4399,7 +4480,7 @@
         <v>45743.390918874728</v>
       </c>
       <c r="G23" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H23" t="s">
         <v>192</v>
@@ -4421,10 +4502,10 @@
         <v>261</v>
       </c>
       <c r="B24" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="C24" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="D24" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4437,7 +4518,7 @@
         <v>45743.390918881109</v>
       </c>
       <c r="G24" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H24" t="s">
         <v>192</v>
@@ -4459,10 +4540,10 @@
         <v>263</v>
       </c>
       <c r="B25" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="C25" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="D25" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4475,7 +4556,7 @@
         <v>45743.390918887373</v>
       </c>
       <c r="G25" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H25" t="s">
         <v>192</v>
@@ -4497,10 +4578,10 @@
         <v>265</v>
       </c>
       <c r="B26" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C26" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="D26" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4513,7 +4594,7 @@
         <v>45743.39091889358</v>
       </c>
       <c r="G26" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H26" t="s">
         <v>192</v>
@@ -4535,10 +4616,10 @@
         <v>267</v>
       </c>
       <c r="B27" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C27" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="D27" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4551,7 +4632,7 @@
         <v>45743.390918900091</v>
       </c>
       <c r="G27" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H27" t="s">
         <v>192</v>
@@ -4573,10 +4654,10 @@
         <v>269</v>
       </c>
       <c r="B28" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C28" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="D28" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4589,7 +4670,7 @@
         <v>45743.390918906553</v>
       </c>
       <c r="G28" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H28" t="s">
         <v>192</v>
@@ -5191,7 +5272,7 @@
         <v>180</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>181</v>
@@ -5212,7 +5293,7 @@
         <v>184</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>185</v>
@@ -5245,7 +5326,7 @@
         <v>nominal1</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E2" s="6" t="str">
         <f>$C2&amp;$D2</f>
@@ -5293,7 +5374,7 @@
         <v>nominal2</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E3" s="6" t="str">
         <f t="shared" ref="E3:E39" si="0">$C3&amp;$D3</f>
@@ -5341,7 +5422,7 @@
         <v>ordinal1</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E4" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5389,7 +5470,7 @@
         <v>ordinal2</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E5" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5437,7 +5518,7 @@
         <v>regex1</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E6" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5485,7 +5566,7 @@
         <v>regex2</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E7" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5533,7 +5614,7 @@
         <v>text1</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E8" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5578,7 +5659,7 @@
         <v>text2</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E9" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5623,7 +5704,7 @@
         <v>org1</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E10" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5668,7 +5749,7 @@
         <v>org2</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E11" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5713,7 +5794,7 @@
         <v>geo1</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E12" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5761,7 +5842,7 @@
         <v>geo1</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E13" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5809,7 +5890,7 @@
         <v>geo1</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E14" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5857,7 +5938,7 @@
         <v>geo1</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E15" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5905,7 +5986,7 @@
         <v>geo2</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E16" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5953,7 +6034,7 @@
         <v>geo2</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E17" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6001,7 +6082,7 @@
         <v>geo2</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E18" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6049,7 +6130,7 @@
         <v>geo2</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E19" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6097,7 +6178,7 @@
         <v>time1</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E20" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6142,7 +6223,7 @@
         <v>time1</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E21" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6187,7 +6268,7 @@
         <v>time1</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E22" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6232,7 +6313,7 @@
         <v>time1</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E23" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6277,7 +6358,7 @@
         <v>time1</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="E24" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6322,7 +6403,7 @@
         <v>time2</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E25" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6367,7 +6448,7 @@
         <v>time2</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E26" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6412,7 +6493,7 @@
         <v>time2</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E27" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6457,7 +6538,7 @@
         <v>time2</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E28" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6502,7 +6583,7 @@
         <v>time2</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="E29" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6547,7 +6628,7 @@
         <v>id1</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E30" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6592,7 +6673,7 @@
         <v>id2</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E31" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6637,7 +6718,7 @@
         <v>number1</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E32" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6682,7 +6763,7 @@
         <v>number1</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E33" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6730,7 +6811,7 @@
         <v>number1</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E34" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6778,7 +6859,7 @@
         <v>number2</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E35" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6823,7 +6904,7 @@
         <v>number2</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6871,7 +6952,7 @@
         <v>number2</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E37" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6919,7 +7000,7 @@
         <v>other1</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E38" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6964,7 +7045,7 @@
         <v>other2</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E39" s="6" t="str">
         <f t="shared" si="0"/>
@@ -7178,7 +7259,7 @@
         <v>111</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>112</v>
@@ -7187,7 +7268,7 @@
         <v>113</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>114</v>
@@ -7384,7 +7465,7 @@
         <v>79</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>80</v>
@@ -7691,7 +7772,7 @@
         <v>58</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>59</v>
@@ -7700,7 +7781,7 @@
         <v>138</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>139</v>
@@ -8261,13 +8342,13 @@
         <v>138</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>140</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>141</v>
@@ -9799,7 +9880,7 @@
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B59" t="s">
         <v>123</v>
@@ -9825,7 +9906,7 @@
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B60" t="s">
         <v>127</v>
@@ -9851,7 +9932,7 @@
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B61" t="s">
         <v>131</v>
@@ -9927,19 +10008,19 @@
         <v>312</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="J1" t="s">
         <v>184</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="L1" s="6" t="s">
+        <v>831</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>832</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>833</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -11253,7 +11334,7 @@
         <v>281</v>
       </c>
       <c r="B1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="C1" t="s">
         <v>282</v>
@@ -11265,64 +11346,64 @@
         <v>283</v>
       </c>
       <c r="F1" s="6" t="s">
+        <v>807</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>808</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>809</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>810</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>811</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>812</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>813</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>814</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>815</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>816</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>817</v>
       </c>
       <c r="P1" t="s">
         <v>138</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="R1" t="s">
         <v>717</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="T1" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="U1" t="s">
         <v>716</v>
       </c>
       <c r="V1" s="6" t="s">
+        <v>788</v>
+      </c>
+      <c r="W1" t="s">
         <v>789</v>
       </c>
-      <c r="W1" t="s">
-        <v>790</v>
-      </c>
       <c r="X1" s="6" t="s">
+        <v>818</v>
+      </c>
+      <c r="Y1" s="6" t="s">
         <v>819</v>
-      </c>
-      <c r="Y1" s="6" t="s">
-        <v>820</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.3">
@@ -11333,7 +11414,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="D2" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($C2,User!$A:$A,0))</f>
@@ -11803,7 +11884,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="D7" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($C7,User!$A:$A,0))</f>
@@ -14379,13 +14460,13 @@
         <v>722</v>
       </c>
       <c r="G1" s="24" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="H1" s="24" t="s">
         <v>283</v>
       </c>
       <c r="I1" s="24" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -14483,16 +14564,16 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="C1" t="s">
         <v>135</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="E1" t="s">
         <v>692</v>
@@ -14501,13 +14582,13 @@
         <v>714</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>283</v>
       </c>
       <c r="I1" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="J1" s="6" t="s">
         <v>723</v>
@@ -14519,40 +14600,40 @@
         <v>720</v>
       </c>
       <c r="M1" s="6" t="s">
+        <v>828</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>843</v>
+      </c>
+      <c r="O1" s="6" t="s">
         <v>829</v>
       </c>
-      <c r="N1" s="6" t="s">
-        <v>844</v>
-      </c>
-      <c r="O1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>830</v>
       </c>
-      <c r="P1" s="6" t="s">
-        <v>831</v>
-      </c>
       <c r="Q1" s="6" t="s">
+        <v>840</v>
+      </c>
+      <c r="R1" s="6" t="s">
         <v>841</v>
       </c>
-      <c r="R1" s="6" t="s">
-        <v>842</v>
-      </c>
       <c r="S1" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="T1" s="6" t="s">
+        <v>850</v>
+      </c>
+      <c r="U1" s="6" t="s">
         <v>851</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>852</v>
       </c>
-      <c r="V1" s="6" t="s">
-        <v>853</v>
-      </c>
       <c r="W1" t="s">
+        <v>845</v>
+      </c>
+      <c r="X1" t="s">
         <v>846</v>
-      </c>
-      <c r="X1" t="s">
-        <v>847</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
@@ -14826,7 +14907,7 @@
         <v>case_type1.ordinal2_1 (ORDINAL;Ordinal_2)</v>
       </c>
       <c r="E5" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="G5" s="6" t="str">
         <f t="shared" si="0"/>
@@ -17206,7 +17287,7 @@
         <v>case_type1.number1_1 (INTERVAL;Age in years, intervals 0, 5, 15, 25, 45, 65)</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="G33" s="6" t="str">
         <f t="shared" si="0"/>
@@ -17291,7 +17372,7 @@
         <v>case_type1.number1_1 (INTERVAL;Age in years, intervals 0, 5, 19, 65)</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="G34" s="6" t="str">
         <f t="shared" si="0"/>
@@ -17461,7 +17542,7 @@
         <v>case_type1.number2_1 (INTERVAL;Age in months, intervals 0, 1, 2, 3)</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="G36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -19161,7 +19242,7 @@
         <v>case_type2.number1_1 (INTERVAL;Age in years, intervals 0, 5, 15, 25, 45, 65)</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="G56" s="6" t="str">
         <f t="shared" si="0"/>
@@ -19246,7 +19327,7 @@
         <v>case_type2.number1_1 (INTERVAL;Age in years, intervals 0, 5, 19, 65)</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="G57" s="6" t="str">
         <f t="shared" si="0"/>
@@ -19478,7 +19559,7 @@
         <v>60</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>61</v>
@@ -19487,7 +19568,7 @@
         <v>135</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>136</v>
@@ -21736,7 +21817,7 @@
       </c>
       <c r="E2" t="str">
         <f>VLOOKUP(D2,User!$A:$D,3,0)</f>
-        <v>org_admin1_1@org1_org</v>
+        <v>org_admin1_1@org1.org</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -21758,7 +21839,7 @@
       </c>
       <c r="E3" t="str">
         <f>VLOOKUP(D3,User!$A:$D,3,0)</f>
-        <v>org_admin2_1@org2_org</v>
+        <v>org_admin2_1@org2.org</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -21780,7 +21861,7 @@
       </c>
       <c r="E4" t="str">
         <f>VLOOKUP(D4,User!$A:$D,3,0)</f>
-        <v>org_admin3_1@org3_org</v>
+        <v>org_admin3_1@org3.org</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -21802,7 +21883,7 @@
       </c>
       <c r="E5" t="str">
         <f>VLOOKUP(D5,User!$A:$D,3,0)</f>
-        <v>org_admin4_1@org4_org</v>
+        <v>org_admin4_1@org4.org</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -21824,7 +21905,7 @@
       </c>
       <c r="E6" t="str">
         <f>VLOOKUP(D6,User!$A:$D,3,0)</f>
-        <v>org_admin5_1@org5_org</v>
+        <v>org_admin5_1@org5.org</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -21871,13 +21952,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
@@ -21895,13 +21976,13 @@
         <v>275</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>276</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="N1" s="7" t="s">
         <v>6</v>
@@ -21919,7 +22000,7 @@
         <v>41</v>
       </c>
       <c r="S1" s="8" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>277</v>
@@ -22718,13 +22799,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
@@ -22739,13 +22820,13 @@
         <v>275</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="K1" s="7" t="s">
         <v>276</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>6</v>
@@ -22760,10 +22841,10 @@
         <v>9</v>
       </c>
       <c r="Q1" s="8" t="s">
+        <v>824</v>
+      </c>
+      <c r="R1" s="8" t="s">
         <v>825</v>
-      </c>
-      <c r="R1" s="8" t="s">
-        <v>826</v>
       </c>
       <c r="S1" s="4" t="s">
         <v>277</v>
@@ -22775,7 +22856,7 @@
         <v>1</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="W1" s="15" t="s">
         <v>284</v>
@@ -23627,13 +23708,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D1" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -23654,19 +23735,19 @@
         <v>213</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="M1" s="6" t="s">
+        <v>824</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>825</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="8" t="s">
         <v>826</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>827</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -23763,13 +23844,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D1" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -23790,13 +23871,13 @@
         <v>213</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="M1" t="s">
         <v>41</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -23876,25 +23957,25 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>858</v>
+      </c>
+      <c r="C1" t="s">
         <v>859</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="6" t="s">
         <v>860</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" t="s">
+        <v>865</v>
+      </c>
+      <c r="F1" t="s">
+        <v>866</v>
+      </c>
+      <c r="G1" t="s">
         <v>861</v>
       </c>
-      <c r="E1" t="s">
-        <v>866</v>
-      </c>
-      <c r="F1" t="s">
-        <v>867</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>862</v>
-      </c>
-      <c r="H1" t="s">
-        <v>863</v>
       </c>
       <c r="I1" t="s">
         <v>416</v>
@@ -23902,7 +23983,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B2" t="s">
         <v>315</v>
@@ -23936,7 +24017,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B3" t="s">
         <v>315</v>
@@ -24105,10 +24186,10 @@
         <v>386</v>
       </c>
       <c r="J1" s="25" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="K1" s="25" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -24473,7 +24554,7 @@
         <v>Municipalities</v>
       </c>
       <c r="D11" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E11" t="s">
         <v>745</v>
@@ -24511,7 +24592,7 @@
         <v>Municipalities</v>
       </c>
       <c r="D12" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="E12" t="s">
         <v>746</v>
@@ -24552,7 +24633,7 @@
         <v>747</v>
       </c>
       <c r="E13" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -24590,7 +24671,7 @@
         <v>748</v>
       </c>
       <c r="E14" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -24628,7 +24709,7 @@
         <v>749</v>
       </c>
       <c r="E15" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -25425,7 +25506,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>190</v>
@@ -25443,19 +25524,19 @@
         <v>41</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>798</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>799</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>800</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>801</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>802</v>
       </c>
       <c r="M1" s="17" t="s">
         <v>285</v>
@@ -25463,13 +25544,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B2" t="s">
-        <v>752</v>
+        <v>874</v>
       </c>
       <c r="C2" t="s">
-        <v>752</v>
+        <v>874</v>
       </c>
       <c r="D2" t="str">
         <f>LEFT(C2,FIND("@",C2)-1)</f>
@@ -25479,7 +25560,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="G2" t="s">
         <v>43</v>
@@ -25514,10 +25595,10 @@
         <v>192</v>
       </c>
       <c r="B3" t="s">
-        <v>753</v>
+        <v>875</v>
       </c>
       <c r="C3" t="s">
-        <v>753</v>
+        <v>875</v>
       </c>
       <c r="D3" t="str">
         <f t="shared" ref="D3:D29" si="0">LEFT(C3,FIND("@",C3)-1)</f>
@@ -25527,7 +25608,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G3" t="s">
         <v>43</v>
@@ -25562,10 +25643,10 @@
         <v>193</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>754</v>
+        <v>876</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>754</v>
+        <v>876</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="0"/>
@@ -25575,7 +25656,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G4" t="s">
         <v>43</v>
@@ -25610,10 +25691,10 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>755</v>
+        <v>877</v>
       </c>
       <c r="C5" t="s">
-        <v>755</v>
+        <v>877</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="0"/>
@@ -25623,7 +25704,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G5" t="s">
         <v>43</v>
@@ -25658,10 +25739,10 @@
         <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>756</v>
+        <v>878</v>
       </c>
       <c r="C6" t="s">
-        <v>756</v>
+        <v>878</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="0"/>
@@ -25671,7 +25752,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G6" t="s">
         <v>46</v>
@@ -25706,10 +25787,10 @@
         <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>757</v>
+        <v>879</v>
       </c>
       <c r="C7" t="s">
-        <v>757</v>
+        <v>879</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="0"/>
@@ -25719,7 +25800,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G7" t="s">
         <v>49</v>
@@ -25754,10 +25835,10 @@
         <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>758</v>
+        <v>880</v>
       </c>
       <c r="C8" t="s">
-        <v>758</v>
+        <v>880</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="0"/>
@@ -25767,7 +25848,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G8" t="s">
         <v>52</v>
@@ -25802,10 +25883,10 @@
         <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>759</v>
+        <v>881</v>
       </c>
       <c r="C9" t="s">
-        <v>759</v>
+        <v>881</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="0"/>
@@ -25815,7 +25896,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G9" t="s">
         <v>55</v>
@@ -25850,10 +25931,10 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>760</v>
+        <v>882</v>
       </c>
       <c r="C10" t="s">
-        <v>760</v>
+        <v>882</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="0"/>
@@ -25863,7 +25944,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G10" t="s">
         <v>43</v>
@@ -25898,10 +25979,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>761</v>
+        <v>883</v>
       </c>
       <c r="C11" t="s">
-        <v>761</v>
+        <v>883</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="0"/>
@@ -25911,7 +25992,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G11" t="s">
         <v>43</v>
@@ -25946,10 +26027,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>762</v>
+        <v>884</v>
       </c>
       <c r="C12" t="s">
-        <v>762</v>
+        <v>884</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="0"/>
@@ -25959,7 +26040,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G12" t="s">
         <v>43</v>
@@ -25994,10 +26075,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>763</v>
+        <v>885</v>
       </c>
       <c r="C13" t="s">
-        <v>763</v>
+        <v>885</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="0"/>
@@ -26007,7 +26088,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G13" t="s">
         <v>43</v>
@@ -26042,10 +26123,10 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>764</v>
+        <v>886</v>
       </c>
       <c r="C14" t="s">
-        <v>764</v>
+        <v>886</v>
       </c>
       <c r="D14" t="str">
         <f t="shared" si="0"/>
@@ -26055,7 +26136,7 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G14" t="s">
         <v>46</v>
@@ -26090,10 +26171,10 @@
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>765</v>
+        <v>887</v>
       </c>
       <c r="C15" t="s">
-        <v>765</v>
+        <v>887</v>
       </c>
       <c r="D15" t="str">
         <f t="shared" si="0"/>
@@ -26103,7 +26184,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G15" t="s">
         <v>46</v>
@@ -26138,10 +26219,10 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>766</v>
+        <v>888</v>
       </c>
       <c r="C16" t="s">
-        <v>766</v>
+        <v>888</v>
       </c>
       <c r="D16" t="str">
         <f t="shared" si="0"/>
@@ -26151,7 +26232,7 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G16" t="s">
         <v>46</v>
@@ -26186,10 +26267,10 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>767</v>
+        <v>889</v>
       </c>
       <c r="C17" t="s">
-        <v>767</v>
+        <v>889</v>
       </c>
       <c r="D17" t="str">
         <f t="shared" si="0"/>
@@ -26199,7 +26280,7 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G17" t="s">
         <v>46</v>
@@ -26234,10 +26315,10 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>768</v>
+        <v>890</v>
       </c>
       <c r="C18" t="s">
-        <v>768</v>
+        <v>890</v>
       </c>
       <c r="D18" t="str">
         <f t="shared" si="0"/>
@@ -26247,7 +26328,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G18" t="s">
         <v>49</v>
@@ -26282,10 +26363,10 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>769</v>
+        <v>891</v>
       </c>
       <c r="C19" t="s">
-        <v>769</v>
+        <v>891</v>
       </c>
       <c r="D19" t="str">
         <f t="shared" si="0"/>
@@ -26295,7 +26376,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G19" t="s">
         <v>49</v>
@@ -26330,10 +26411,10 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>770</v>
+        <v>892</v>
       </c>
       <c r="C20" t="s">
-        <v>770</v>
+        <v>892</v>
       </c>
       <c r="D20" t="str">
         <f t="shared" si="0"/>
@@ -26343,7 +26424,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G20" t="s">
         <v>49</v>
@@ -26378,10 +26459,10 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>771</v>
+        <v>893</v>
       </c>
       <c r="C21" t="s">
-        <v>771</v>
+        <v>893</v>
       </c>
       <c r="D21" t="str">
         <f t="shared" si="0"/>
@@ -26391,7 +26472,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G21" t="s">
         <v>49</v>
@@ -26426,10 +26507,10 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>772</v>
+        <v>894</v>
       </c>
       <c r="C22" t="s">
-        <v>772</v>
+        <v>894</v>
       </c>
       <c r="D22" t="str">
         <f t="shared" si="0"/>
@@ -26439,7 +26520,7 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G22" t="s">
         <v>52</v>
@@ -26474,10 +26555,10 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>773</v>
+        <v>895</v>
       </c>
       <c r="C23" t="s">
-        <v>773</v>
+        <v>895</v>
       </c>
       <c r="D23" t="str">
         <f t="shared" si="0"/>
@@ -26487,7 +26568,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G23" t="s">
         <v>52</v>
@@ -26522,10 +26603,10 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>774</v>
+        <v>896</v>
       </c>
       <c r="C24" t="s">
-        <v>774</v>
+        <v>896</v>
       </c>
       <c r="D24" t="str">
         <f t="shared" si="0"/>
@@ -26535,7 +26616,7 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G24" t="s">
         <v>52</v>
@@ -26570,10 +26651,10 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>775</v>
+        <v>897</v>
       </c>
       <c r="C25" t="s">
-        <v>775</v>
+        <v>897</v>
       </c>
       <c r="D25" t="str">
         <f t="shared" si="0"/>
@@ -26583,7 +26664,7 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G25" t="s">
         <v>52</v>
@@ -26618,10 +26699,10 @@
         <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>776</v>
+        <v>898</v>
       </c>
       <c r="C26" t="s">
-        <v>776</v>
+        <v>898</v>
       </c>
       <c r="D26" t="str">
         <f t="shared" si="0"/>
@@ -26631,7 +26712,7 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G26" t="s">
         <v>55</v>
@@ -26666,10 +26747,10 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>777</v>
+        <v>899</v>
       </c>
       <c r="C27" t="s">
-        <v>777</v>
+        <v>899</v>
       </c>
       <c r="D27" t="str">
         <f t="shared" si="0"/>
@@ -26679,7 +26760,7 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G27" t="s">
         <v>55</v>
@@ -26714,10 +26795,10 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>778</v>
+        <v>900</v>
       </c>
       <c r="C28" t="s">
-        <v>778</v>
+        <v>900</v>
       </c>
       <c r="D28" t="str">
         <f t="shared" si="0"/>
@@ -26727,7 +26808,7 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G28" t="s">
         <v>55</v>
@@ -26762,10 +26843,10 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>779</v>
+        <v>901</v>
       </c>
       <c r="C29" t="s">
-        <v>779</v>
+        <v>901</v>
       </c>
       <c r="D29" t="str">
         <f t="shared" si="0"/>
@@ -26775,7 +26856,7 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G29" t="s">
         <v>55</v>
@@ -26807,8 +26888,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="refdata_admin1_1@org1.org" xr:uid="{6720259D-8B8B-404B-BBFC-255A858BC201}"/>
-    <hyperlink ref="B4" r:id="rId2" display="refdata_admin1_1@org1.org" xr:uid="{20728C37-5C65-48C8-8BFF-B78EF176652E}"/>
+    <hyperlink ref="C4" r:id="rId1" xr:uid="{6720259D-8B8B-404B-BBFC-255A858BC201}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{20728C37-5C65-48C8-8BFF-B78EF176652E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: root user creation updated to use key claim instead of id to identify if exists or not (#220)
* fix: root user creation updated to use key claim instead of id to identify if exists or not

* refactor: commondb UserManager create_root_user_from_claims updated
refactor: removed root user id from toml

---------

Co-authored-by: Ivo van Walle <ivo.van.walle@rivm.nl>
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F5C3440-E169-49AB-B04F-4AB419B33125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B50F3BB1-41BD-43FD-8DD5-18F1B5FB645A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3552" yWindow="3552" windowWidth="30960" windowHeight="12120" tabRatio="913" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4248" yWindow="4248" windowWidth="30960" windowHeight="12120" tabRatio="913" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="875">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="902">
   <si>
     <t>id</t>
   </si>
@@ -2380,9 +2380,6 @@
     <t>to_region_name</t>
   </si>
   <si>
-    <t>root1_1@org1_org</t>
-  </si>
-  <si>
     <t>app_admin1_1@org1_org</t>
   </si>
   <si>
@@ -2747,6 +2744,90 @@
   </si>
   <si>
     <t>["CASEDB_ROOT"]</t>
+  </si>
+  <si>
+    <t>root1_1@org1.org</t>
+  </si>
+  <si>
+    <t>app_admin1_1@org1.org</t>
+  </si>
+  <si>
+    <t>refdata_admin1_1@org1.org</t>
+  </si>
+  <si>
+    <t>org_admin1_1@org1.org</t>
+  </si>
+  <si>
+    <t>org_admin2_1@org2.org</t>
+  </si>
+  <si>
+    <t>org_admin3_1@org3.org</t>
+  </si>
+  <si>
+    <t>org_admin4_1@org4.org</t>
+  </si>
+  <si>
+    <t>org_admin5_1@org5.org</t>
+  </si>
+  <si>
+    <t>org_user1_1@org1.org</t>
+  </si>
+  <si>
+    <t>org_user1_2@org1.org</t>
+  </si>
+  <si>
+    <t>org_user1_3@org1.org</t>
+  </si>
+  <si>
+    <t>org_user1_4@org1.org</t>
+  </si>
+  <si>
+    <t>org_user2_1@org2.org</t>
+  </si>
+  <si>
+    <t>org_user2_2@org2.org</t>
+  </si>
+  <si>
+    <t>org_user2_3@org2.org</t>
+  </si>
+  <si>
+    <t>org_user2_4@org2.org</t>
+  </si>
+  <si>
+    <t>org_user3_1@org3.org</t>
+  </si>
+  <si>
+    <t>org_user3_2@org3.org</t>
+  </si>
+  <si>
+    <t>org_user3_3@org3.org</t>
+  </si>
+  <si>
+    <t>org_user3_4@org3.org</t>
+  </si>
+  <si>
+    <t>org_user4_1@org4.org</t>
+  </si>
+  <si>
+    <t>org_user4_2@org4.org</t>
+  </si>
+  <si>
+    <t>org_user4_3@org4.org</t>
+  </si>
+  <si>
+    <t>org_user4_4@org4.org</t>
+  </si>
+  <si>
+    <t>org_user5_1@org5.org</t>
+  </si>
+  <si>
+    <t>org_user5_2@org5.org</t>
+  </si>
+  <si>
+    <t>org_user5_3@org5.org</t>
+  </si>
+  <si>
+    <t>org_user5_4@org5.org</t>
   </si>
 </sst>
 </file>
@@ -3550,7 +3631,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>190</v>
@@ -3585,10 +3666,10 @@
         <v>217</v>
       </c>
       <c r="B2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="C2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="D2" s="6" t="str">
         <f>LEFT($C2,LEN($C2)-9)</f>
@@ -3601,10 +3682,10 @@
         <v>45743.390918726589</v>
       </c>
       <c r="G2" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="H2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="I2" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($H2,User!$A:$A,0))</f>
@@ -3623,10 +3704,10 @@
         <v>219</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="D3" s="6" t="str">
         <f t="shared" ref="D3:D28" si="0">LEFT($C3,LEN($C3)-9)</f>
@@ -3639,7 +3720,7 @@
         <v>45743.390918741461</v>
       </c>
       <c r="G3" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="H3" t="s">
         <v>192</v>
@@ -3661,10 +3742,10 @@
         <v>221</v>
       </c>
       <c r="B4" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="C4" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="D4" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3677,7 +3758,7 @@
         <v>45743.390918746562</v>
       </c>
       <c r="G4" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H4" t="s">
         <v>192</v>
@@ -3699,10 +3780,10 @@
         <v>223</v>
       </c>
       <c r="B5" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="C5" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="D5" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3715,7 +3796,7 @@
         <v>45743.390918763551</v>
       </c>
       <c r="G5" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H5" t="s">
         <v>192</v>
@@ -3737,10 +3818,10 @@
         <v>225</v>
       </c>
       <c r="B6" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C6" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="D6" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3753,7 +3834,7 @@
         <v>45743.390918772537</v>
       </c>
       <c r="G6" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H6" t="s">
         <v>192</v>
@@ -3775,10 +3856,10 @@
         <v>227</v>
       </c>
       <c r="B7" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C7" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="D7" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3791,7 +3872,7 @@
         <v>45743.390918781181</v>
       </c>
       <c r="G7" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H7" t="s">
         <v>192</v>
@@ -3813,10 +3894,10 @@
         <v>229</v>
       </c>
       <c r="B8" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="C8" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="D8" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3829,7 +3910,7 @@
         <v>45743.3909187889</v>
       </c>
       <c r="G8" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="H8" t="s">
         <v>192</v>
@@ -3851,10 +3932,10 @@
         <v>231</v>
       </c>
       <c r="B9" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="C9" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="D9" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3867,7 +3948,7 @@
         <v>45743.390918796598</v>
       </c>
       <c r="G9" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H9" t="s">
         <v>192</v>
@@ -3889,10 +3970,10 @@
         <v>233</v>
       </c>
       <c r="B10" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="C10" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="D10" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3905,7 +3986,7 @@
         <v>45743.390918801953</v>
       </c>
       <c r="G10" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H10" t="s">
         <v>192</v>
@@ -3927,10 +4008,10 @@
         <v>235</v>
       </c>
       <c r="B11" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="C11" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D11" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3943,7 +4024,7 @@
         <v>45743.390918807163</v>
       </c>
       <c r="G11" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H11" t="s">
         <v>192</v>
@@ -3965,10 +4046,10 @@
         <v>237</v>
       </c>
       <c r="B12" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="C12" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="D12" s="6" t="str">
         <f t="shared" si="0"/>
@@ -3981,7 +4062,7 @@
         <v>45743.3909188123</v>
       </c>
       <c r="G12" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H12" t="s">
         <v>192</v>
@@ -4003,10 +4084,10 @@
         <v>239</v>
       </c>
       <c r="B13" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="C13" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="D13" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4019,7 +4100,7 @@
         <v>45743.390918817633</v>
       </c>
       <c r="G13" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H13" t="s">
         <v>192</v>
@@ -4041,10 +4122,10 @@
         <v>241</v>
       </c>
       <c r="B14" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="C14" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="D14" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4057,7 +4138,7 @@
         <v>45743.390918822908</v>
       </c>
       <c r="G14" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H14" t="s">
         <v>192</v>
@@ -4079,10 +4160,10 @@
         <v>243</v>
       </c>
       <c r="B15" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="C15" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="D15" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4095,7 +4176,7 @@
         <v>45743.390918828743</v>
       </c>
       <c r="G15" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H15" t="s">
         <v>192</v>
@@ -4117,10 +4198,10 @@
         <v>245</v>
       </c>
       <c r="B16" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C16" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="D16" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4133,7 +4214,7 @@
         <v>45743.390918834302</v>
       </c>
       <c r="G16" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H16" t="s">
         <v>192</v>
@@ -4155,10 +4236,10 @@
         <v>247</v>
       </c>
       <c r="B17" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C17" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="D17" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4171,7 +4252,7 @@
         <v>45743.390918839839</v>
       </c>
       <c r="G17" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H17" t="s">
         <v>192</v>
@@ -4193,10 +4274,10 @@
         <v>249</v>
       </c>
       <c r="B18" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="C18" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="D18" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4209,7 +4290,7 @@
         <v>45743.390918845187</v>
       </c>
       <c r="G18" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H18" t="s">
         <v>192</v>
@@ -4231,10 +4312,10 @@
         <v>251</v>
       </c>
       <c r="B19" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C19" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="D19" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4247,7 +4328,7 @@
         <v>45743.390918851088</v>
       </c>
       <c r="G19" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H19" t="s">
         <v>192</v>
@@ -4269,10 +4350,10 @@
         <v>253</v>
       </c>
       <c r="B20" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C20" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="D20" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4285,7 +4366,7 @@
         <v>45743.39091885696</v>
       </c>
       <c r="G20" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H20" t="s">
         <v>192</v>
@@ -4307,10 +4388,10 @@
         <v>255</v>
       </c>
       <c r="B21" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="C21" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="D21" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4323,7 +4404,7 @@
         <v>45743.390918862962</v>
       </c>
       <c r="G21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H21" t="s">
         <v>192</v>
@@ -4345,10 +4426,10 @@
         <v>257</v>
       </c>
       <c r="B22" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="C22" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D22" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4361,7 +4442,7 @@
         <v>45743.390918868739</v>
       </c>
       <c r="G22" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H22" t="s">
         <v>192</v>
@@ -4383,10 +4464,10 @@
         <v>259</v>
       </c>
       <c r="B23" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="C23" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="D23" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4399,7 +4480,7 @@
         <v>45743.390918874728</v>
       </c>
       <c r="G23" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H23" t="s">
         <v>192</v>
@@ -4421,10 +4502,10 @@
         <v>261</v>
       </c>
       <c r="B24" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="C24" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="D24" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4437,7 +4518,7 @@
         <v>45743.390918881109</v>
       </c>
       <c r="G24" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H24" t="s">
         <v>192</v>
@@ -4459,10 +4540,10 @@
         <v>263</v>
       </c>
       <c r="B25" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="C25" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="D25" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4475,7 +4556,7 @@
         <v>45743.390918887373</v>
       </c>
       <c r="G25" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H25" t="s">
         <v>192</v>
@@ -4497,10 +4578,10 @@
         <v>265</v>
       </c>
       <c r="B26" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C26" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="D26" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4513,7 +4594,7 @@
         <v>45743.39091889358</v>
       </c>
       <c r="G26" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H26" t="s">
         <v>192</v>
@@ -4535,10 +4616,10 @@
         <v>267</v>
       </c>
       <c r="B27" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C27" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="D27" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4551,7 +4632,7 @@
         <v>45743.390918900091</v>
       </c>
       <c r="G27" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H27" t="s">
         <v>192</v>
@@ -4573,10 +4654,10 @@
         <v>269</v>
       </c>
       <c r="B28" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C28" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="D28" s="6" t="str">
         <f t="shared" si="0"/>
@@ -4589,7 +4670,7 @@
         <v>45743.390918906553</v>
       </c>
       <c r="G28" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="H28" t="s">
         <v>192</v>
@@ -5191,7 +5272,7 @@
         <v>180</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>181</v>
@@ -5212,7 +5293,7 @@
         <v>184</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>185</v>
@@ -5245,7 +5326,7 @@
         <v>nominal1</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E2" s="6" t="str">
         <f>$C2&amp;$D2</f>
@@ -5293,7 +5374,7 @@
         <v>nominal2</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E3" s="6" t="str">
         <f t="shared" ref="E3:E39" si="0">$C3&amp;$D3</f>
@@ -5341,7 +5422,7 @@
         <v>ordinal1</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E4" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5389,7 +5470,7 @@
         <v>ordinal2</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E5" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5437,7 +5518,7 @@
         <v>regex1</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E6" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5485,7 +5566,7 @@
         <v>regex2</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E7" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5533,7 +5614,7 @@
         <v>text1</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E8" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5578,7 +5659,7 @@
         <v>text2</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E9" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5623,7 +5704,7 @@
         <v>org1</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E10" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5668,7 +5749,7 @@
         <v>org2</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E11" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5713,7 +5794,7 @@
         <v>geo1</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E12" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5761,7 +5842,7 @@
         <v>geo1</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E13" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5809,7 +5890,7 @@
         <v>geo1</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E14" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5857,7 +5938,7 @@
         <v>geo1</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E15" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5905,7 +5986,7 @@
         <v>geo2</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E16" s="6" t="str">
         <f t="shared" si="0"/>
@@ -5953,7 +6034,7 @@
         <v>geo2</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E17" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6001,7 +6082,7 @@
         <v>geo2</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E18" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6049,7 +6130,7 @@
         <v>geo2</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E19" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6097,7 +6178,7 @@
         <v>time1</v>
       </c>
       <c r="D20" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E20" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6142,7 +6223,7 @@
         <v>time1</v>
       </c>
       <c r="D21" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E21" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6187,7 +6268,7 @@
         <v>time1</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E22" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6232,7 +6313,7 @@
         <v>time1</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E23" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6277,7 +6358,7 @@
         <v>time1</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="E24" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6322,7 +6403,7 @@
         <v>time2</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E25" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6367,7 +6448,7 @@
         <v>time2</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="E26" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6412,7 +6493,7 @@
         <v>time2</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="E27" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6457,7 +6538,7 @@
         <v>time2</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="E28" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6502,7 +6583,7 @@
         <v>time2</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="E29" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6547,7 +6628,7 @@
         <v>id1</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E30" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6592,7 +6673,7 @@
         <v>id2</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E31" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6637,7 +6718,7 @@
         <v>number1</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E32" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6682,7 +6763,7 @@
         <v>number1</v>
       </c>
       <c r="D33" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E33" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6730,7 +6811,7 @@
         <v>number1</v>
       </c>
       <c r="D34" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E34" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6778,7 +6859,7 @@
         <v>number2</v>
       </c>
       <c r="D35" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E35" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6823,7 +6904,7 @@
         <v>number2</v>
       </c>
       <c r="D36" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6871,7 +6952,7 @@
         <v>number2</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E37" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6919,7 +7000,7 @@
         <v>other1</v>
       </c>
       <c r="D38" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E38" s="6" t="str">
         <f t="shared" si="0"/>
@@ -6964,7 +7045,7 @@
         <v>other2</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="E39" s="6" t="str">
         <f t="shared" si="0"/>
@@ -7178,7 +7259,7 @@
         <v>111</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>112</v>
@@ -7187,7 +7268,7 @@
         <v>113</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>114</v>
@@ -7384,7 +7465,7 @@
         <v>79</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>80</v>
@@ -7691,7 +7772,7 @@
         <v>58</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>59</v>
@@ -7700,7 +7781,7 @@
         <v>138</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>139</v>
@@ -8261,13 +8342,13 @@
         <v>138</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>140</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>141</v>
@@ -9799,7 +9880,7 @@
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="B59" t="s">
         <v>123</v>
@@ -9825,7 +9906,7 @@
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B60" t="s">
         <v>127</v>
@@ -9851,7 +9932,7 @@
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B61" t="s">
         <v>131</v>
@@ -9927,19 +10008,19 @@
         <v>312</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="J1" t="s">
         <v>184</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="L1" s="6" t="s">
+        <v>831</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>832</v>
-      </c>
-      <c r="M1" s="6" t="s">
-        <v>833</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -11253,7 +11334,7 @@
         <v>281</v>
       </c>
       <c r="B1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="C1" t="s">
         <v>282</v>
@@ -11265,64 +11346,64 @@
         <v>283</v>
       </c>
       <c r="F1" s="6" t="s">
+        <v>807</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>808</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>809</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>810</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>811</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>812</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>813</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>814</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>815</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>816</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>817</v>
       </c>
       <c r="P1" t="s">
         <v>138</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="R1" t="s">
         <v>717</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="T1" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="U1" t="s">
         <v>716</v>
       </c>
       <c r="V1" s="6" t="s">
+        <v>788</v>
+      </c>
+      <c r="W1" t="s">
         <v>789</v>
       </c>
-      <c r="W1" t="s">
-        <v>790</v>
-      </c>
       <c r="X1" s="6" t="s">
+        <v>818</v>
+      </c>
+      <c r="Y1" s="6" t="s">
         <v>819</v>
-      </c>
-      <c r="Y1" s="6" t="s">
-        <v>820</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.3">
@@ -11333,7 +11414,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="D2" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($C2,User!$A:$A,0))</f>
@@ -11803,7 +11884,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="D7" s="6" t="str">
         <f>INDEX(User!$D:$D,MATCH($C7,User!$A:$A,0))</f>
@@ -14379,13 +14460,13 @@
         <v>722</v>
       </c>
       <c r="G1" s="24" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="H1" s="24" t="s">
         <v>283</v>
       </c>
       <c r="I1" s="24" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -14483,16 +14564,16 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="C1" t="s">
         <v>135</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="E1" t="s">
         <v>692</v>
@@ -14501,13 +14582,13 @@
         <v>714</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>283</v>
       </c>
       <c r="I1" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="J1" s="6" t="s">
         <v>723</v>
@@ -14519,40 +14600,40 @@
         <v>720</v>
       </c>
       <c r="M1" s="6" t="s">
+        <v>828</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>843</v>
+      </c>
+      <c r="O1" s="6" t="s">
         <v>829</v>
       </c>
-      <c r="N1" s="6" t="s">
-        <v>844</v>
-      </c>
-      <c r="O1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>830</v>
       </c>
-      <c r="P1" s="6" t="s">
-        <v>831</v>
-      </c>
       <c r="Q1" s="6" t="s">
+        <v>840</v>
+      </c>
+      <c r="R1" s="6" t="s">
         <v>841</v>
       </c>
-      <c r="R1" s="6" t="s">
-        <v>842</v>
-      </c>
       <c r="S1" s="6" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="T1" s="6" t="s">
+        <v>850</v>
+      </c>
+      <c r="U1" s="6" t="s">
         <v>851</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>852</v>
       </c>
-      <c r="V1" s="6" t="s">
-        <v>853</v>
-      </c>
       <c r="W1" t="s">
+        <v>845</v>
+      </c>
+      <c r="X1" t="s">
         <v>846</v>
-      </c>
-      <c r="X1" t="s">
-        <v>847</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
@@ -14826,7 +14907,7 @@
         <v>case_type1.ordinal2_1 (ORDINAL;Ordinal_2)</v>
       </c>
       <c r="E5" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="G5" s="6" t="str">
         <f t="shared" si="0"/>
@@ -17206,7 +17287,7 @@
         <v>case_type1.number1_1 (INTERVAL;Age in years, intervals 0, 5, 15, 25, 45, 65)</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="G33" s="6" t="str">
         <f t="shared" si="0"/>
@@ -17291,7 +17372,7 @@
         <v>case_type1.number1_1 (INTERVAL;Age in years, intervals 0, 5, 19, 65)</v>
       </c>
       <c r="E34" s="11" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="G34" s="6" t="str">
         <f t="shared" si="0"/>
@@ -17461,7 +17542,7 @@
         <v>case_type1.number2_1 (INTERVAL;Age in months, intervals 0, 1, 2, 3)</v>
       </c>
       <c r="E36" s="11" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="G36" s="6" t="str">
         <f t="shared" si="0"/>
@@ -19161,7 +19242,7 @@
         <v>case_type2.number1_1 (INTERVAL;Age in years, intervals 0, 5, 15, 25, 45, 65)</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="G56" s="6" t="str">
         <f t="shared" si="0"/>
@@ -19246,7 +19327,7 @@
         <v>case_type2.number1_1 (INTERVAL;Age in years, intervals 0, 5, 19, 65)</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="G57" s="6" t="str">
         <f t="shared" si="0"/>
@@ -19478,7 +19559,7 @@
         <v>60</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>61</v>
@@ -19487,7 +19568,7 @@
         <v>135</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>136</v>
@@ -21736,7 +21817,7 @@
       </c>
       <c r="E2" t="str">
         <f>VLOOKUP(D2,User!$A:$D,3,0)</f>
-        <v>org_admin1_1@org1_org</v>
+        <v>org_admin1_1@org1.org</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -21758,7 +21839,7 @@
       </c>
       <c r="E3" t="str">
         <f>VLOOKUP(D3,User!$A:$D,3,0)</f>
-        <v>org_admin2_1@org2_org</v>
+        <v>org_admin2_1@org2.org</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -21780,7 +21861,7 @@
       </c>
       <c r="E4" t="str">
         <f>VLOOKUP(D4,User!$A:$D,3,0)</f>
-        <v>org_admin3_1@org3_org</v>
+        <v>org_admin3_1@org3.org</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -21802,7 +21883,7 @@
       </c>
       <c r="E5" t="str">
         <f>VLOOKUP(D5,User!$A:$D,3,0)</f>
-        <v>org_admin4_1@org4_org</v>
+        <v>org_admin4_1@org4.org</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -21824,7 +21905,7 @@
       </c>
       <c r="E6" t="str">
         <f>VLOOKUP(D6,User!$A:$D,3,0)</f>
-        <v>org_admin5_1@org5_org</v>
+        <v>org_admin5_1@org5.org</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -21871,13 +21952,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
@@ -21895,13 +21976,13 @@
         <v>275</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>276</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="N1" s="7" t="s">
         <v>6</v>
@@ -21919,7 +22000,7 @@
         <v>41</v>
       </c>
       <c r="S1" s="8" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="T1" s="4" t="s">
         <v>277</v>
@@ -22718,13 +22799,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
@@ -22739,13 +22820,13 @@
         <v>275</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="K1" s="7" t="s">
         <v>276</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="M1" s="7" t="s">
         <v>6</v>
@@ -22760,10 +22841,10 @@
         <v>9</v>
       </c>
       <c r="Q1" s="8" t="s">
+        <v>824</v>
+      </c>
+      <c r="R1" s="8" t="s">
         <v>825</v>
-      </c>
-      <c r="R1" s="8" t="s">
-        <v>826</v>
       </c>
       <c r="S1" s="4" t="s">
         <v>277</v>
@@ -22775,7 +22856,7 @@
         <v>1</v>
       </c>
       <c r="V1" s="8" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="W1" s="15" t="s">
         <v>284</v>
@@ -23627,13 +23708,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D1" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -23654,19 +23735,19 @@
         <v>213</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="M1" s="6" t="s">
+        <v>824</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>825</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="8" t="s">
         <v>826</v>
-      </c>
-      <c r="O1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>827</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -23763,13 +23844,13 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="D1" t="s">
         <v>58</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -23790,13 +23871,13 @@
         <v>213</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="M1" t="s">
         <v>41</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
@@ -23876,25 +23957,25 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>858</v>
+      </c>
+      <c r="C1" t="s">
         <v>859</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="6" t="s">
         <v>860</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" t="s">
+        <v>865</v>
+      </c>
+      <c r="F1" t="s">
+        <v>866</v>
+      </c>
+      <c r="G1" t="s">
         <v>861</v>
       </c>
-      <c r="E1" t="s">
-        <v>866</v>
-      </c>
-      <c r="F1" t="s">
-        <v>867</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>862</v>
-      </c>
-      <c r="H1" t="s">
-        <v>863</v>
       </c>
       <c r="I1" t="s">
         <v>416</v>
@@ -23902,7 +23983,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B2" t="s">
         <v>315</v>
@@ -23936,7 +24017,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B3" t="s">
         <v>315</v>
@@ -24105,10 +24186,10 @@
         <v>386</v>
       </c>
       <c r="J1" s="25" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="K1" s="25" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -24473,7 +24554,7 @@
         <v>Municipalities</v>
       </c>
       <c r="D11" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="E11" t="s">
         <v>745</v>
@@ -24511,7 +24592,7 @@
         <v>Municipalities</v>
       </c>
       <c r="D12" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="E12" t="s">
         <v>746</v>
@@ -24552,7 +24633,7 @@
         <v>747</v>
       </c>
       <c r="E13" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="F13">
         <v>1</v>
@@ -24590,7 +24671,7 @@
         <v>748</v>
       </c>
       <c r="E14" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -24628,7 +24709,7 @@
         <v>749</v>
       </c>
       <c r="E15" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -25425,7 +25506,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>190</v>
@@ -25443,19 +25524,19 @@
         <v>41</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>798</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>799</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>800</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>801</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>802</v>
       </c>
       <c r="M1" s="17" t="s">
         <v>285</v>
@@ -25463,13 +25544,13 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B2" t="s">
-        <v>752</v>
+        <v>874</v>
       </c>
       <c r="C2" t="s">
-        <v>752</v>
+        <v>874</v>
       </c>
       <c r="D2" t="str">
         <f>LEFT(C2,FIND("@",C2)-1)</f>
@@ -25479,7 +25560,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="G2" t="s">
         <v>43</v>
@@ -25514,10 +25595,10 @@
         <v>192</v>
       </c>
       <c r="B3" t="s">
-        <v>753</v>
+        <v>875</v>
       </c>
       <c r="C3" t="s">
-        <v>753</v>
+        <v>875</v>
       </c>
       <c r="D3" t="str">
         <f t="shared" ref="D3:D29" si="0">LEFT(C3,FIND("@",C3)-1)</f>
@@ -25527,7 +25608,7 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="G3" t="s">
         <v>43</v>
@@ -25562,10 +25643,10 @@
         <v>193</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>754</v>
+        <v>876</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>754</v>
+        <v>876</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" si="0"/>
@@ -25575,7 +25656,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="G4" t="s">
         <v>43</v>
@@ -25610,10 +25691,10 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>755</v>
+        <v>877</v>
       </c>
       <c r="C5" t="s">
-        <v>755</v>
+        <v>877</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="0"/>
@@ -25623,7 +25704,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G5" t="s">
         <v>43</v>
@@ -25658,10 +25739,10 @@
         <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>756</v>
+        <v>878</v>
       </c>
       <c r="C6" t="s">
-        <v>756</v>
+        <v>878</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="0"/>
@@ -25671,7 +25752,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G6" t="s">
         <v>46</v>
@@ -25706,10 +25787,10 @@
         <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>757</v>
+        <v>879</v>
       </c>
       <c r="C7" t="s">
-        <v>757</v>
+        <v>879</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="0"/>
@@ -25719,7 +25800,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G7" t="s">
         <v>49</v>
@@ -25754,10 +25835,10 @@
         <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>758</v>
+        <v>880</v>
       </c>
       <c r="C8" t="s">
-        <v>758</v>
+        <v>880</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="0"/>
@@ -25767,7 +25848,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G8" t="s">
         <v>52</v>
@@ -25802,10 +25883,10 @@
         <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>759</v>
+        <v>881</v>
       </c>
       <c r="C9" t="s">
-        <v>759</v>
+        <v>881</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="0"/>
@@ -25815,7 +25896,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="G9" t="s">
         <v>55</v>
@@ -25850,10 +25931,10 @@
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>760</v>
+        <v>882</v>
       </c>
       <c r="C10" t="s">
-        <v>760</v>
+        <v>882</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="0"/>
@@ -25863,7 +25944,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G10" t="s">
         <v>43</v>
@@ -25898,10 +25979,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>761</v>
+        <v>883</v>
       </c>
       <c r="C11" t="s">
-        <v>761</v>
+        <v>883</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="0"/>
@@ -25911,7 +25992,7 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G11" t="s">
         <v>43</v>
@@ -25946,10 +26027,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>762</v>
+        <v>884</v>
       </c>
       <c r="C12" t="s">
-        <v>762</v>
+        <v>884</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="0"/>
@@ -25959,7 +26040,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G12" t="s">
         <v>43</v>
@@ -25994,10 +26075,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>763</v>
+        <v>885</v>
       </c>
       <c r="C13" t="s">
-        <v>763</v>
+        <v>885</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="0"/>
@@ -26007,7 +26088,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G13" t="s">
         <v>43</v>
@@ -26042,10 +26123,10 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>764</v>
+        <v>886</v>
       </c>
       <c r="C14" t="s">
-        <v>764</v>
+        <v>886</v>
       </c>
       <c r="D14" t="str">
         <f t="shared" si="0"/>
@@ -26055,7 +26136,7 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G14" t="s">
         <v>46</v>
@@ -26090,10 +26171,10 @@
         <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>765</v>
+        <v>887</v>
       </c>
       <c r="C15" t="s">
-        <v>765</v>
+        <v>887</v>
       </c>
       <c r="D15" t="str">
         <f t="shared" si="0"/>
@@ -26103,7 +26184,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G15" t="s">
         <v>46</v>
@@ -26138,10 +26219,10 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>766</v>
+        <v>888</v>
       </c>
       <c r="C16" t="s">
-        <v>766</v>
+        <v>888</v>
       </c>
       <c r="D16" t="str">
         <f t="shared" si="0"/>
@@ -26151,7 +26232,7 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G16" t="s">
         <v>46</v>
@@ -26186,10 +26267,10 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>767</v>
+        <v>889</v>
       </c>
       <c r="C17" t="s">
-        <v>767</v>
+        <v>889</v>
       </c>
       <c r="D17" t="str">
         <f t="shared" si="0"/>
@@ -26199,7 +26280,7 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G17" t="s">
         <v>46</v>
@@ -26234,10 +26315,10 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>768</v>
+        <v>890</v>
       </c>
       <c r="C18" t="s">
-        <v>768</v>
+        <v>890</v>
       </c>
       <c r="D18" t="str">
         <f t="shared" si="0"/>
@@ -26247,7 +26328,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G18" t="s">
         <v>49</v>
@@ -26282,10 +26363,10 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>769</v>
+        <v>891</v>
       </c>
       <c r="C19" t="s">
-        <v>769</v>
+        <v>891</v>
       </c>
       <c r="D19" t="str">
         <f t="shared" si="0"/>
@@ -26295,7 +26376,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G19" t="s">
         <v>49</v>
@@ -26330,10 +26411,10 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>770</v>
+        <v>892</v>
       </c>
       <c r="C20" t="s">
-        <v>770</v>
+        <v>892</v>
       </c>
       <c r="D20" t="str">
         <f t="shared" si="0"/>
@@ -26343,7 +26424,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G20" t="s">
         <v>49</v>
@@ -26378,10 +26459,10 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>771</v>
+        <v>893</v>
       </c>
       <c r="C21" t="s">
-        <v>771</v>
+        <v>893</v>
       </c>
       <c r="D21" t="str">
         <f t="shared" si="0"/>
@@ -26391,7 +26472,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G21" t="s">
         <v>49</v>
@@ -26426,10 +26507,10 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>772</v>
+        <v>894</v>
       </c>
       <c r="C22" t="s">
-        <v>772</v>
+        <v>894</v>
       </c>
       <c r="D22" t="str">
         <f t="shared" si="0"/>
@@ -26439,7 +26520,7 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G22" t="s">
         <v>52</v>
@@ -26474,10 +26555,10 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>773</v>
+        <v>895</v>
       </c>
       <c r="C23" t="s">
-        <v>773</v>
+        <v>895</v>
       </c>
       <c r="D23" t="str">
         <f t="shared" si="0"/>
@@ -26487,7 +26568,7 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G23" t="s">
         <v>52</v>
@@ -26522,10 +26603,10 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>774</v>
+        <v>896</v>
       </c>
       <c r="C24" t="s">
-        <v>774</v>
+        <v>896</v>
       </c>
       <c r="D24" t="str">
         <f t="shared" si="0"/>
@@ -26535,7 +26616,7 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G24" t="s">
         <v>52</v>
@@ -26570,10 +26651,10 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>775</v>
+        <v>897</v>
       </c>
       <c r="C25" t="s">
-        <v>775</v>
+        <v>897</v>
       </c>
       <c r="D25" t="str">
         <f t="shared" si="0"/>
@@ -26583,7 +26664,7 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G25" t="s">
         <v>52</v>
@@ -26618,10 +26699,10 @@
         <v>34</v>
       </c>
       <c r="B26" t="s">
-        <v>776</v>
+        <v>898</v>
       </c>
       <c r="C26" t="s">
-        <v>776</v>
+        <v>898</v>
       </c>
       <c r="D26" t="str">
         <f t="shared" si="0"/>
@@ -26631,7 +26712,7 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G26" t="s">
         <v>55</v>
@@ -26666,10 +26747,10 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>777</v>
+        <v>899</v>
       </c>
       <c r="C27" t="s">
-        <v>777</v>
+        <v>899</v>
       </c>
       <c r="D27" t="str">
         <f t="shared" si="0"/>
@@ -26679,7 +26760,7 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G27" t="s">
         <v>55</v>
@@ -26714,10 +26795,10 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>778</v>
+        <v>900</v>
       </c>
       <c r="C28" t="s">
-        <v>778</v>
+        <v>900</v>
       </c>
       <c r="D28" t="str">
         <f t="shared" si="0"/>
@@ -26727,7 +26808,7 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G28" t="s">
         <v>55</v>
@@ -26762,10 +26843,10 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>779</v>
+        <v>901</v>
       </c>
       <c r="C29" t="s">
-        <v>779</v>
+        <v>901</v>
       </c>
       <c r="D29" t="str">
         <f t="shared" si="0"/>
@@ -26775,7 +26856,7 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="G29" t="s">
         <v>55</v>
@@ -26807,8 +26888,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="refdata_admin1_1@org1.org" xr:uid="{6720259D-8B8B-404B-BBFC-255A858BC201}"/>
-    <hyperlink ref="B4" r:id="rId2" display="refdata_admin1_1@org1.org" xr:uid="{20728C37-5C65-48C8-8BFF-B78EF176652E}"/>
+    <hyperlink ref="C4" r:id="rId1" xr:uid="{6720259D-8B8B-404B-BBFC-255A858BC201}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{20728C37-5C65-48C8-8BFF-B78EF176652E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test: minor test fixes
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B50F3BB1-41BD-43FD-8DD5-18F1B5FB645A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15D68C03-77B7-465F-9F92-AB1E5B601812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4248" yWindow="4248" windowWidth="30960" windowHeight="12120" tabRatio="913" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2467" uniqueCount="903">
   <si>
     <t>id</t>
   </si>
@@ -2828,6 +2828,9 @@
   </si>
   <si>
     <t>org_user5_4@org5.org</t>
+  </si>
+  <si>
+    <t>resolution</t>
   </si>
 </sst>
 </file>
@@ -24056,16 +24059,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26B8A4C3-472B-45B0-ABE1-5F12E28FD147}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="53.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.109375" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -24075,11 +24079,14 @@
       <c r="C1" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="1" t="s">
+        <v>902</v>
+      </c>
+      <c r="E1" s="21" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>387</v>
       </c>
@@ -24089,11 +24096,14 @@
       <c r="C2" t="s">
         <v>377</v>
       </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>388</v>
       </c>
@@ -24103,11 +24113,14 @@
       <c r="C3" t="s">
         <v>378</v>
       </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>389</v>
       </c>
@@ -24117,11 +24130,14 @@
       <c r="C4" t="s">
         <v>379</v>
       </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>390</v>
       </c>
@@ -24131,7 +24147,10 @@
       <c r="C5" t="s">
         <v>380</v>
       </c>
-      <c r="D5" t="b">
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: minor test fixes (#252)
Co-authored-by: MarkStreek <mvdstreek2003@gmail.com>
Co-authored-by: Ivo van Walle <ivo.van.walle@rivm.nl>
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B50F3BB1-41BD-43FD-8DD5-18F1B5FB645A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15D68C03-77B7-465F-9F92-AB1E5B601812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4248" yWindow="4248" windowWidth="30960" windowHeight="12120" tabRatio="913" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2467" uniqueCount="903">
   <si>
     <t>id</t>
   </si>
@@ -2828,6 +2828,9 @@
   </si>
   <si>
     <t>org_user5_4@org5.org</t>
+  </si>
+  <si>
+    <t>resolution</t>
   </si>
 </sst>
 </file>
@@ -24056,16 +24059,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26B8A4C3-472B-45B0-ABE1-5F12E28FD147}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="53.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.109375" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -24075,11 +24079,14 @@
       <c r="C1" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="1" t="s">
+        <v>902</v>
+      </c>
+      <c r="E1" s="21" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>387</v>
       </c>
@@ -24089,11 +24096,14 @@
       <c r="C2" t="s">
         <v>377</v>
       </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>388</v>
       </c>
@@ -24103,11 +24113,14 @@
       <c r="C3" t="s">
         <v>378</v>
       </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>389</v>
       </c>
@@ -24117,11 +24130,14 @@
       <c r="C4" t="s">
         <v>379</v>
       </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>390</v>
       </c>
@@ -24131,7 +24147,10 @@
       <c r="C5" t="s">
         <v>380</v>
       </c>
-      <c r="D5" t="b">
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "chore(deps): update dependency python to v3.14.1 (#174)"
This reverts commit da1c1a6261914624105c8002211a5de9263b3a93.
</commit_message>
<xml_diff>
--- a/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
+++ b/test/casedb/integration/case_validation/test_casedb_case_validation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivo_v\Documents\gen-epix-api\test\casedb\integration\case_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15D68C03-77B7-465F-9F92-AB1E5B601812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B50F3BB1-41BD-43FD-8DD5-18F1B5FB645A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" tabRatio="913" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4248" yWindow="4248" windowWidth="30960" windowHeight="12120" tabRatio="913" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ConceptSet" sheetId="30" r:id="rId1"/>
@@ -122,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2467" uniqueCount="903">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="902">
   <si>
     <t>id</t>
   </si>
@@ -2828,9 +2828,6 @@
   </si>
   <si>
     <t>org_user5_4@org5.org</t>
-  </si>
-  <si>
-    <t>resolution</t>
   </si>
 </sst>
 </file>
@@ -24059,17 +24056,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26B8A4C3-472B-45B0-ABE1-5F12E28FD147}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="53.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.109375" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -24079,14 +24075,11 @@
       <c r="C1" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>902</v>
-      </c>
-      <c r="E1" s="21" t="s">
+      <c r="D1" s="21" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>387</v>
       </c>
@@ -24096,14 +24089,11 @@
       <c r="C2" t="s">
         <v>377</v>
       </c>
-      <c r="D2">
-        <v>4</v>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>388</v>
       </c>
@@ -24113,14 +24103,11 @@
       <c r="C3" t="s">
         <v>378</v>
       </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>389</v>
       </c>
@@ -24130,14 +24117,11 @@
       <c r="C4" t="s">
         <v>379</v>
       </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>390</v>
       </c>
@@ -24147,10 +24131,7 @@
       <c r="C5" t="s">
         <v>380</v>
       </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5" t="b">
+      <c r="D5" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>